<commit_message>
Nebius: scheduled go-live quarters so the model holds both 2026 guidance ranges; campuses and regional queues
Nebius: the register may schedule single quarters (mw_added_2026q3 = 50, mw_added_2026q4 = 350,
both proposed); the flat pace covers the rest. 2026 revenue lands at 3.3 USD bn (guidance 3.0 to
3.4) with year-end ARR of 8.6 USD bn (guidance 7 to 9); a straight-line ramp gave 3.8. The plan
row on the Drivers sheet is pasted from the register. Write-up and table updated.

Stack: stack/campuses.csv (six AI campuses, planned and operating MW each with its own source);
eight regional interconnection-queue rows from LBNL's Queued Up 2026 (they sum to the 2,061 GW
total).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/NBIS.xlsx
+++ b/models/NBIS.xlsx
@@ -34,6 +34,8 @@
     <definedName name="in_arr_guidance_ye2026_high_usd_m">Inputs!$B$17</definedName>
     <definedName name="in_revenue_guidance_2026_low_usd_m">Inputs!$B$18</definedName>
     <definedName name="in_revenue_guidance_2026_high_usd_m">Inputs!$B$19</definedName>
+    <definedName name="in_mw_added_2026q3">Inputs!$B$20</definedName>
+    <definedName name="in_mw_added_2026q4">Inputs!$B$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -64,10 +66,10 @@
       <color rgb="00595959"/>
     </font>
     <font>
-      <color rgb="00008000"/>
+      <color rgb="00000000"/>
     </font>
     <font>
-      <color rgb="00000000"/>
+      <color rgb="00008000"/>
     </font>
     <font>
       <b val="1"/>
@@ -115,8 +117,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,12 +128,12 @@
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -723,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1202,6 +1204,56 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mw_added_2026q3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>6-K EX-99.2 2026-05-13 and 2026-08-12 (2026 revenue guidance 3.0 to 3.4 USD bn; ARR guidance 7 to 9 USD bn; capacity added in Q3 to expand the footprint)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>[derived; proposed; range 25 to 200] Active power going live in Q3 2026, overriding the flat pace for this quarter. The company guides to 3.0 to 3.4 USD bn of 2026 revenue and 7 to 9 USD bn of ARR at year end. With 981 USD m booked in the first half, both hold only if little new capacity bills in Q3 and most of it arrives in Q4: 200 MW in each quarter gives 3.8 USD bn of revenue, above the range, while 50 then 350 gives 3.3 USD bn and the same 8.6 USD bn of ARR. The split is inferred from the guidance, not disclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mw_added_2026q4</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>6-K EX-99.2 2026-05-13 and 2026-08-12 (800 MW to 1 GW connected by end 2026)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>[derived; proposed; range 200 to 500] Active power going live in Q4 2026, overriding the flat pace for this quarter; see mw_added_2026q3. Takes active power from 350 MW to 700 MW at December 2026, inside the 800 MW to 1 GW of connected power the company expects by then.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1213,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1331,7 +1383,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Active power, end of quarter (disclosed Dec 2025; June 2026 inferred from ARR)</t>
+          <t>Active power going live, plan (register: mw_added_&lt;quarter&gt; where given, else mw_added_per_quarter)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1342,58 +1394,44 @@
       <c r="C2" s="13" t="n"/>
       <c r="D2" s="13" t="n"/>
       <c r="E2" s="13" t="n"/>
-      <c r="F2" s="13" t="n">
-        <v>170</v>
-      </c>
+      <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
-      <c r="H2" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="I2" s="14">
-        <f>H2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="J2" s="14">
-        <f>I2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="K2" s="14">
-        <f>J2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="L2" s="14">
-        <f>K2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="M2" s="14">
-        <f>L2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="N2" s="14">
-        <f>M2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="O2" s="14">
-        <f>N2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="P2" s="14">
-        <f>O2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="Q2" s="14">
-        <f>P2+in_mw_added_per_quarter</f>
-        <v/>
-      </c>
-      <c r="R2" s="14">
-        <f>Q2+in_mw_added_per_quarter</f>
-        <v/>
+      <c r="H2" s="13" t="n"/>
+      <c r="I2" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="J2" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="K2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="L2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="M2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="N2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="O2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="P2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="Q2" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="R2" s="13" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Active power added (went live)</t>
+          <t>Active power, end of quarter (disclosed Dec 2025; June 2026 inferred from ARR)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1404,54 +1442,58 @@
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
-      <c r="F3" s="13" t="n"/>
+      <c r="F3" s="13" t="n">
+        <v>170</v>
+      </c>
       <c r="G3" s="13" t="n"/>
-      <c r="H3" s="13" t="n"/>
-      <c r="I3" s="15">
-        <f>I2-H2</f>
-        <v/>
-      </c>
-      <c r="J3" s="15">
-        <f>J2-I2</f>
-        <v/>
-      </c>
-      <c r="K3" s="15">
-        <f>K2-J2</f>
-        <v/>
-      </c>
-      <c r="L3" s="15">
-        <f>L2-K2</f>
-        <v/>
-      </c>
-      <c r="M3" s="15">
-        <f>M2-L2</f>
-        <v/>
-      </c>
-      <c r="N3" s="15">
-        <f>N2-M2</f>
-        <v/>
-      </c>
-      <c r="O3" s="15">
-        <f>O2-N2</f>
-        <v/>
-      </c>
-      <c r="P3" s="15">
-        <f>P2-O2</f>
-        <v/>
-      </c>
-      <c r="Q3" s="15">
-        <f>Q2-P2</f>
-        <v/>
-      </c>
-      <c r="R3" s="15">
-        <f>R2-Q2</f>
+      <c r="H3" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="I3" s="14">
+        <f>H3+I2</f>
+        <v/>
+      </c>
+      <c r="J3" s="14">
+        <f>I3+J2</f>
+        <v/>
+      </c>
+      <c r="K3" s="14">
+        <f>J3+K2</f>
+        <v/>
+      </c>
+      <c r="L3" s="14">
+        <f>K3+L2</f>
+        <v/>
+      </c>
+      <c r="M3" s="14">
+        <f>L3+M2</f>
+        <v/>
+      </c>
+      <c r="N3" s="14">
+        <f>M3+N2</f>
+        <v/>
+      </c>
+      <c r="O3" s="14">
+        <f>N3+O2</f>
+        <v/>
+      </c>
+      <c r="P3" s="14">
+        <f>O3+P2</f>
+        <v/>
+      </c>
+      <c r="Q3" s="14">
+        <f>P3+Q2</f>
+        <v/>
+      </c>
+      <c r="R3" s="14">
+        <f>Q3+R2</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Active power, average</t>
+          <t>Active power added (went live)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1465,121 +1507,109 @@
       <c r="F4" s="13" t="n"/>
       <c r="G4" s="13" t="n"/>
       <c r="H4" s="13" t="n"/>
-      <c r="I4" s="15">
-        <f>(H2+I2)/2</f>
-        <v/>
-      </c>
-      <c r="J4" s="15">
-        <f>(I2+J2)/2</f>
-        <v/>
-      </c>
-      <c r="K4" s="15">
-        <f>(J2+K2)/2</f>
-        <v/>
-      </c>
-      <c r="L4" s="15">
-        <f>(K2+L2)/2</f>
-        <v/>
-      </c>
-      <c r="M4" s="15">
-        <f>(L2+M2)/2</f>
-        <v/>
-      </c>
-      <c r="N4" s="15">
-        <f>(M2+N2)/2</f>
-        <v/>
-      </c>
-      <c r="O4" s="15">
-        <f>(N2+O2)/2</f>
-        <v/>
-      </c>
-      <c r="P4" s="15">
-        <f>(O2+P2)/2</f>
-        <v/>
-      </c>
-      <c r="Q4" s="15">
-        <f>(P2+Q2)/2</f>
-        <v/>
-      </c>
-      <c r="R4" s="15">
-        <f>(Q2+R2)/2</f>
+      <c r="I4" s="14">
+        <f>I3-H3</f>
+        <v/>
+      </c>
+      <c r="J4" s="14">
+        <f>J3-I3</f>
+        <v/>
+      </c>
+      <c r="K4" s="14">
+        <f>K3-J3</f>
+        <v/>
+      </c>
+      <c r="L4" s="14">
+        <f>L3-K3</f>
+        <v/>
+      </c>
+      <c r="M4" s="14">
+        <f>M3-L3</f>
+        <v/>
+      </c>
+      <c r="N4" s="14">
+        <f>N3-M3</f>
+        <v/>
+      </c>
+      <c r="O4" s="14">
+        <f>O3-N3</f>
+        <v/>
+      </c>
+      <c r="P4" s="14">
+        <f>P3-O3</f>
+        <v/>
+      </c>
+      <c r="Q4" s="14">
+        <f>Q3-P3</f>
+        <v/>
+      </c>
+      <c r="R4" s="14">
+        <f>R3-Q3</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Annualised run-rate revenue (ARR), end of quarter</t>
+          <t>Active power, average</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>USD m</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>249</v>
-      </c>
-      <c r="D5" s="16" t="n">
-        <v>430</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>551</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G5" s="16" t="n">
-        <v>1900</v>
-      </c>
-      <c r="H5" s="16" t="n">
-        <v>3000</v>
-      </c>
-      <c r="I5" s="17">
-        <f>H5+I3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="J5" s="17">
-        <f>I5+J3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="K5" s="17">
-        <f>J5+K3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="L5" s="17">
-        <f>K5+L3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="M5" s="17">
-        <f>L5+M3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="N5" s="17">
-        <f>M5+N3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="O5" s="17">
-        <f>N5+O3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="P5" s="17">
-        <f>O5+P3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="Q5" s="17">
-        <f>P5+Q3*in_arr_per_new_mw_year_usd_m</f>
-        <v/>
-      </c>
-      <c r="R5" s="17">
-        <f>Q5+R3*in_arr_per_new_mw_year_usd_m</f>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="n"/>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="14">
+        <f>(H3+I3)/2</f>
+        <v/>
+      </c>
+      <c r="J5" s="14">
+        <f>(I3+J3)/2</f>
+        <v/>
+      </c>
+      <c r="K5" s="14">
+        <f>(J3+K3)/2</f>
+        <v/>
+      </c>
+      <c r="L5" s="14">
+        <f>(K3+L3)/2</f>
+        <v/>
+      </c>
+      <c r="M5" s="14">
+        <f>(L3+M3)/2</f>
+        <v/>
+      </c>
+      <c r="N5" s="14">
+        <f>(M3+N3)/2</f>
+        <v/>
+      </c>
+      <c r="O5" s="14">
+        <f>(N3+O3)/2</f>
+        <v/>
+      </c>
+      <c r="P5" s="14">
+        <f>(O3+P3)/2</f>
+        <v/>
+      </c>
+      <c r="Q5" s="14">
+        <f>(P3+Q3)/2</f>
+        <v/>
+      </c>
+      <c r="R5" s="14">
+        <f>(Q3+R3)/2</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AI cloud revenue</t>
+          <t>Annualised run-rate revenue (ARR), end of quarter</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1587,63 +1617,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n">
-        <v>214.2</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>389.7</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>574.9</v>
-      </c>
-      <c r="I6" s="17">
-        <f>(H5+I5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="J6" s="17">
-        <f>(I5+J5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="K6" s="17">
-        <f>(J5+K5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="L6" s="17">
-        <f>(K5+L5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="M6" s="17">
-        <f>(L5+M5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="N6" s="17">
-        <f>(M5+N5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="O6" s="17">
-        <f>(N5+O5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="P6" s="17">
-        <f>(O5+P5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="Q6" s="17">
-        <f>(P5+Q5)/8*in_revenue_to_midpoint_arr</f>
-        <v/>
-      </c>
-      <c r="R6" s="17">
-        <f>(Q5+R5)/8*in_revenue_to_midpoint_arr</f>
+      <c r="C6" s="15" t="n">
+        <v>249</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>430</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>551</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>1900</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I6" s="16">
+        <f>H6+I4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="J6" s="16">
+        <f>I6+J4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="K6" s="16">
+        <f>J6+K4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="L6" s="16">
+        <f>K6+L4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="M6" s="16">
+        <f>L6+M4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="N6" s="16">
+        <f>M6+N4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="O6" s="16">
+        <f>N6+O4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="P6" s="16">
+        <f>O6+P4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="Q6" s="16">
+        <f>P6+Q4*in_arr_per_new_mw_year_usd_m</f>
+        <v/>
+      </c>
+      <c r="R6" s="16">
+        <f>Q6+R4*in_arr_per_new_mw_year_usd_m</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Revenue, group</t>
+          <t>AI cloud revenue</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1651,69 +1687,63 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n">
-        <v>55.3</v>
-      </c>
-      <c r="D7" s="16" t="n">
-        <v>105.1</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>146.1</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <v>227.7</v>
-      </c>
-      <c r="G7" s="16" t="n">
-        <v>399</v>
-      </c>
-      <c r="H7" s="16" t="n">
-        <v>582.3</v>
-      </c>
-      <c r="I7" s="17">
-        <f>I6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="J7" s="17">
-        <f>J6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="K7" s="17">
-        <f>K6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="L7" s="17">
-        <f>L6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="M7" s="17">
-        <f>M6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="N7" s="17">
-        <f>N6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="O7" s="17">
-        <f>O6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="P7" s="17">
-        <f>P6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="Q7" s="17">
-        <f>Q6/in_ai_cloud_share_of_revenue</f>
-        <v/>
-      </c>
-      <c r="R7" s="17">
-        <f>R6/in_ai_cloud_share_of_revenue</f>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n">
+        <v>214.2</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>389.7</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>574.9</v>
+      </c>
+      <c r="I7" s="16">
+        <f>(H6+I6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="J7" s="16">
+        <f>(I6+J6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="K7" s="16">
+        <f>(J6+K6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="L7" s="16">
+        <f>(K6+L6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="M7" s="16">
+        <f>(L6+M6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="N7" s="16">
+        <f>(M6+N6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="O7" s="16">
+        <f>(N6+O6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="P7" s="16">
+        <f>(O6+P6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="Q7" s="16">
+        <f>(P6+Q6)/8*in_revenue_to_midpoint_arr</f>
+        <v/>
+      </c>
+      <c r="R7" s="16">
+        <f>(Q6+R6)/8*in_revenue_to_midpoint_arr</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Adjusted EBITDA, group</t>
+          <t>Revenue, group</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1721,69 +1751,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
-        <v>-62.6</v>
-      </c>
-      <c r="D8" s="16" t="n">
-        <v>-21</v>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="F8" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>129.5</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <v>236.2</v>
-      </c>
-      <c r="I8" s="17">
-        <f>I7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="J8" s="17">
-        <f>J7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="K8" s="17">
-        <f>K7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="L8" s="17">
-        <f>L7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="M8" s="17">
-        <f>M7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="N8" s="17">
-        <f>N7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="O8" s="17">
-        <f>O7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="P8" s="17">
-        <f>P7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="Q8" s="17">
-        <f>Q7*in_adjusted_ebitda_margin</f>
-        <v/>
-      </c>
-      <c r="R8" s="17">
-        <f>R7*in_adjusted_ebitda_margin</f>
+      <c r="C8" s="15" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>146.1</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>227.7</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>399</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>582.3</v>
+      </c>
+      <c r="I8" s="16">
+        <f>I7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="J8" s="16">
+        <f>J7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="K8" s="16">
+        <f>K7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="L8" s="16">
+        <f>L7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="M8" s="16">
+        <f>M7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="N8" s="16">
+        <f>N7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="O8" s="16">
+        <f>O7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="P8" s="16">
+        <f>P7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="Q8" s="16">
+        <f>Q7/in_ai_cloud_share_of_revenue</f>
+        <v/>
+      </c>
+      <c r="R8" s="16">
+        <f>R7/in_ai_cloud_share_of_revenue</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Capital expenditure</t>
+          <t>Adjusted EBITDA, group</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1791,69 +1821,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
-        <v>543.9</v>
-      </c>
-      <c r="D9" s="16" t="n">
-        <v>510.6</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>955.5</v>
-      </c>
-      <c r="F9" s="16" t="n">
-        <v>2056</v>
-      </c>
-      <c r="G9" s="16" t="n">
-        <v>2472.9</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>5657.4</v>
-      </c>
-      <c r="I9" s="17">
-        <f>in_capex_per_mw_usd_m*I3</f>
-        <v/>
-      </c>
-      <c r="J9" s="17">
-        <f>in_capex_per_mw_usd_m*J3</f>
-        <v/>
-      </c>
-      <c r="K9" s="17">
-        <f>in_capex_per_mw_usd_m*K3</f>
-        <v/>
-      </c>
-      <c r="L9" s="17">
-        <f>in_capex_per_mw_usd_m*L3</f>
-        <v/>
-      </c>
-      <c r="M9" s="17">
-        <f>in_capex_per_mw_usd_m*M3</f>
-        <v/>
-      </c>
-      <c r="N9" s="17">
-        <f>in_capex_per_mw_usd_m*N3</f>
-        <v/>
-      </c>
-      <c r="O9" s="17">
-        <f>in_capex_per_mw_usd_m*O3</f>
-        <v/>
-      </c>
-      <c r="P9" s="17">
-        <f>in_capex_per_mw_usd_m*P3</f>
-        <v/>
-      </c>
-      <c r="Q9" s="17">
-        <f>in_capex_per_mw_usd_m*Q3</f>
-        <v/>
-      </c>
-      <c r="R9" s="17">
-        <f>in_capex_per_mw_usd_m*R3</f>
+      <c r="C9" s="15" t="n">
+        <v>-62.6</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>-21</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>236.2</v>
+      </c>
+      <c r="I9" s="16">
+        <f>I8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>J8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="K9" s="16">
+        <f>K8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="L9" s="16">
+        <f>L8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="M9" s="16">
+        <f>M8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="N9" s="16">
+        <f>N8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="O9" s="16">
+        <f>O8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="P9" s="16">
+        <f>P8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="Q9" s="16">
+        <f>Q8*in_adjusted_ebitda_margin</f>
+        <v/>
+      </c>
+      <c r="R9" s="16">
+        <f>R8*in_adjusted_ebitda_margin</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Customer prepayments received</t>
+          <t>Capital expenditure</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1861,57 +1891,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="16" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="16" t="n"/>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
-      <c r="I10" s="17">
-        <f>I9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="J10" s="17">
-        <f>J9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="K10" s="17">
-        <f>K9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="L10" s="17">
-        <f>L9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="M10" s="17">
-        <f>M9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="N10" s="17">
-        <f>N9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="O10" s="17">
-        <f>O9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="P10" s="17">
-        <f>P9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="Q10" s="17">
-        <f>Q9*in_prepayment_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="R10" s="17">
-        <f>R9*in_prepayment_share_of_capex</f>
+      <c r="C10" s="15" t="n">
+        <v>543.9</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>510.6</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>955.5</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>2056</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>2472.9</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>5657.4</v>
+      </c>
+      <c r="I10" s="16">
+        <f>in_capex_per_mw_usd_m*I4</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>in_capex_per_mw_usd_m*J4</f>
+        <v/>
+      </c>
+      <c r="K10" s="16">
+        <f>in_capex_per_mw_usd_m*K4</f>
+        <v/>
+      </c>
+      <c r="L10" s="16">
+        <f>in_capex_per_mw_usd_m*L4</f>
+        <v/>
+      </c>
+      <c r="M10" s="16">
+        <f>in_capex_per_mw_usd_m*M4</f>
+        <v/>
+      </c>
+      <c r="N10" s="16">
+        <f>in_capex_per_mw_usd_m*N4</f>
+        <v/>
+      </c>
+      <c r="O10" s="16">
+        <f>in_capex_per_mw_usd_m*O4</f>
+        <v/>
+      </c>
+      <c r="P10" s="16">
+        <f>in_capex_per_mw_usd_m*P4</f>
+        <v/>
+      </c>
+      <c r="Q10" s="16">
+        <f>in_capex_per_mw_usd_m*Q4</f>
+        <v/>
+      </c>
+      <c r="R10" s="16">
+        <f>in_capex_per_mw_usd_m*R4</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prepaid revenue recognised (non-cash)</t>
+          <t>Customer prepayments received</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1919,57 +1961,57 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="17">
-        <f>H14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="J11" s="17">
-        <f>I14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="K11" s="17">
-        <f>J14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="L11" s="17">
-        <f>K14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="M11" s="17">
-        <f>L14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="N11" s="17">
-        <f>M14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="O11" s="17">
-        <f>N14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="P11" s="17">
-        <f>O14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="Q11" s="17">
-        <f>P14*in_prepaid_revenue_recognised_share_per_quarter</f>
-        <v/>
-      </c>
-      <c r="R11" s="17">
-        <f>Q14*in_prepaid_revenue_recognised_share_per_quarter</f>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="16">
+        <f>I10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>J10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="K11" s="16">
+        <f>K10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="L11" s="16">
+        <f>L10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="M11" s="16">
+        <f>M10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="N11" s="16">
+        <f>N10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="O11" s="16">
+        <f>O10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="P11" s="16">
+        <f>P10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="Q11" s="16">
+        <f>Q10*in_prepayment_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="R11" s="16">
+        <f>R10*in_prepayment_share_of_capex</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Change in deferred revenue (cash flow statement)</t>
+          <t>Prepaid revenue recognised (non-cash)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1977,69 +2019,57 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C12" s="16" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D12" s="16" t="n">
-        <v>0.3000000000000007</v>
-      </c>
-      <c r="E12" s="16" t="n">
-        <v>-3.8</v>
-      </c>
-      <c r="F12" s="16" t="n">
-        <v>1566.5</v>
-      </c>
-      <c r="G12" s="16" t="n">
-        <v>3198</v>
-      </c>
-      <c r="H12" s="16" t="n">
-        <v>1197</v>
-      </c>
-      <c r="I12" s="18">
-        <f>I10-I11</f>
-        <v/>
-      </c>
-      <c r="J12" s="18">
-        <f>J10-J11</f>
-        <v/>
-      </c>
-      <c r="K12" s="18">
-        <f>K10-K11</f>
-        <v/>
-      </c>
-      <c r="L12" s="18">
-        <f>L10-L11</f>
-        <v/>
-      </c>
-      <c r="M12" s="18">
-        <f>M10-M11</f>
-        <v/>
-      </c>
-      <c r="N12" s="18">
-        <f>N10-N11</f>
-        <v/>
-      </c>
-      <c r="O12" s="18">
-        <f>O10-O11</f>
-        <v/>
-      </c>
-      <c r="P12" s="18">
-        <f>P10-P11</f>
-        <v/>
-      </c>
-      <c r="Q12" s="18">
-        <f>Q10-Q11</f>
-        <v/>
-      </c>
-      <c r="R12" s="18">
-        <f>R10-R11</f>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="16">
+        <f>H15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="J12" s="16">
+        <f>I15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="K12" s="16">
+        <f>J15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="L12" s="16">
+        <f>K15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="M12" s="16">
+        <f>L15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="N12" s="16">
+        <f>M15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="O12" s="16">
+        <f>N15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="P12" s="16">
+        <f>O15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="Q12" s="16">
+        <f>P15*in_prepaid_revenue_recognised_share_per_quarter</f>
+        <v/>
+      </c>
+      <c r="R12" s="16">
+        <f>Q15*in_prepaid_revenue_recognised_share_per_quarter</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Other deferred revenue movements (plug to reported balance)</t>
+          <t>Change in deferred revenue (cash flow statement)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2047,59 +2077,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>0.09999999999999876</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>-4.599999999999909</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>2.600000000000364</v>
-      </c>
-      <c r="H13" s="16" t="n">
-        <v>0.0999999999994543</v>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="16" t="n">
-        <v>0</v>
+      <c r="C13" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>0.3000000000000007</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>1566.5</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>3198</v>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>1197</v>
+      </c>
+      <c r="I13" s="17">
+        <f>I11-I12</f>
+        <v/>
+      </c>
+      <c r="J13" s="17">
+        <f>J11-J12</f>
+        <v/>
+      </c>
+      <c r="K13" s="17">
+        <f>K11-K12</f>
+        <v/>
+      </c>
+      <c r="L13" s="17">
+        <f>L11-L12</f>
+        <v/>
+      </c>
+      <c r="M13" s="17">
+        <f>M11-M12</f>
+        <v/>
+      </c>
+      <c r="N13" s="17">
+        <f>N11-N12</f>
+        <v/>
+      </c>
+      <c r="O13" s="17">
+        <f>O11-O12</f>
+        <v/>
+      </c>
+      <c r="P13" s="17">
+        <f>P11-P12</f>
+        <v/>
+      </c>
+      <c r="Q13" s="17">
+        <f>Q11-Q12</f>
+        <v/>
+      </c>
+      <c r="R13" s="17">
+        <f>R11-R12</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Deferred revenue, end of quarter</t>
+          <t>Other deferred revenue movements (plug to reported balance)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2107,69 +2147,59 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
-        <v>19</v>
-      </c>
-      <c r="D14" s="16" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="E14" s="16" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="F14" s="16" t="n">
-        <v>1577.5</v>
-      </c>
-      <c r="G14" s="16" t="n">
-        <v>4778.1</v>
-      </c>
-      <c r="H14" s="16" t="n">
-        <v>5975.2</v>
-      </c>
-      <c r="I14" s="18">
-        <f>H14+I12+I13</f>
-        <v/>
-      </c>
-      <c r="J14" s="18">
-        <f>I14+J12+J13</f>
-        <v/>
-      </c>
-      <c r="K14" s="18">
-        <f>J14+K12+K13</f>
-        <v/>
-      </c>
-      <c r="L14" s="18">
-        <f>K14+L12+L13</f>
-        <v/>
-      </c>
-      <c r="M14" s="18">
-        <f>L14+M12+M13</f>
-        <v/>
-      </c>
-      <c r="N14" s="18">
-        <f>M14+N12+N13</f>
-        <v/>
-      </c>
-      <c r="O14" s="18">
-        <f>N14+O12+O13</f>
-        <v/>
-      </c>
-      <c r="P14" s="18">
-        <f>O14+P12+P13</f>
-        <v/>
-      </c>
-      <c r="Q14" s="18">
-        <f>P14+Q12+Q13</f>
-        <v/>
-      </c>
-      <c r="R14" s="18">
-        <f>Q14+R12+R13</f>
-        <v/>
+      <c r="C14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.09999999999999876</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>-4.599999999999909</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>2.600000000000364</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.0999999999994543</v>
+      </c>
+      <c r="I14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Interest on debt (inside other items in actuals)</t>
+          <t>Deferred revenue, end of quarter</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2177,57 +2207,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C15" s="16" t="n"/>
-      <c r="D15" s="16" t="n"/>
-      <c r="E15" s="16" t="n"/>
-      <c r="F15" s="16" t="n"/>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="16" t="n"/>
+      <c r="C15" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>1577.5</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>4778.1</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>5975.2</v>
+      </c>
       <c r="I15" s="17">
-        <f>(H19+I19)/2*in_cost_of_debt/4</f>
+        <f>H15+I13+I14</f>
         <v/>
       </c>
       <c r="J15" s="17">
-        <f>(I19+J19)/2*in_cost_of_debt/4</f>
+        <f>I15+J13+J14</f>
         <v/>
       </c>
       <c r="K15" s="17">
-        <f>(J19+K19)/2*in_cost_of_debt/4</f>
+        <f>J15+K13+K14</f>
         <v/>
       </c>
       <c r="L15" s="17">
-        <f>(K19+L19)/2*in_cost_of_debt/4</f>
+        <f>K15+L13+L14</f>
         <v/>
       </c>
       <c r="M15" s="17">
-        <f>(L19+M19)/2*in_cost_of_debt/4</f>
+        <f>L15+M13+M14</f>
         <v/>
       </c>
       <c r="N15" s="17">
-        <f>(M19+N19)/2*in_cost_of_debt/4</f>
+        <f>M15+N13+N14</f>
         <v/>
       </c>
       <c r="O15" s="17">
-        <f>(N19+O19)/2*in_cost_of_debt/4</f>
+        <f>N15+O13+O14</f>
         <v/>
       </c>
       <c r="P15" s="17">
-        <f>(O19+P19)/2*in_cost_of_debt/4</f>
+        <f>O15+P13+P14</f>
         <v/>
       </c>
       <c r="Q15" s="17">
-        <f>(P19+Q19)/2*in_cost_of_debt/4</f>
+        <f>P15+Q13+Q14</f>
         <v/>
       </c>
       <c r="R15" s="17">
-        <f>(Q19+R19)/2*in_cost_of_debt/4</f>
+        <f>Q15+R13+R14</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Other operating cash items (actuals: everything between EBITDA plus deferred revenue and reported cash from operations)</t>
+          <t>Interest on debt (inside other items in actuals)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2235,69 +2277,57 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C16" s="16" t="n">
-        <v>-124</v>
-      </c>
-      <c r="D16" s="16" t="n">
-        <v>-147.2</v>
-      </c>
-      <c r="E16" s="16" t="n">
-        <v>-71.59999999999999</v>
-      </c>
-      <c r="F16" s="16" t="n">
-        <v>-747.2</v>
-      </c>
-      <c r="G16" s="16" t="n">
-        <v>-1069.5</v>
-      </c>
-      <c r="H16" s="16" t="n">
-        <v>812.8999999999999</v>
-      </c>
-      <c r="I16" s="17">
-        <f>I9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="J16" s="17">
-        <f>J9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="K16" s="17">
-        <f>K9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="L16" s="17">
-        <f>L9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="M16" s="17">
-        <f>M9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="N16" s="17">
-        <f>N9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="O16" s="17">
-        <f>O9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="P16" s="17">
-        <f>P9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="Q16" s="17">
-        <f>Q9*in_other_operating_cash_share_of_capex</f>
-        <v/>
-      </c>
-      <c r="R16" s="17">
-        <f>R9*in_other_operating_cash_share_of_capex</f>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="16">
+        <f>(H20+I20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="J16" s="16">
+        <f>(I20+J20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="K16" s="16">
+        <f>(J20+K20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="L16" s="16">
+        <f>(K20+L20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="M16" s="16">
+        <f>(L20+M20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="N16" s="16">
+        <f>(M20+N20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="O16" s="16">
+        <f>(N20+O20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="P16" s="16">
+        <f>(O20+P20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="Q16" s="16">
+        <f>(P20+Q20)/2*in_cost_of_debt/4</f>
+        <v/>
+      </c>
+      <c r="R16" s="16">
+        <f>(Q20+R20)/2*in_cost_of_debt/4</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cash from operations</t>
+          <t>Other operating cash items (actuals: everything between EBITDA plus deferred revenue and reported cash from operations)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2305,69 +2335,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C17" s="16" t="n">
-        <v>-184.1</v>
-      </c>
-      <c r="D17" s="16" t="n">
-        <v>-167.9</v>
-      </c>
-      <c r="E17" s="16" t="n">
-        <v>-80.59999999999999</v>
-      </c>
-      <c r="F17" s="16" t="n">
-        <v>834.3</v>
-      </c>
-      <c r="G17" s="16" t="n">
-        <v>2258</v>
-      </c>
-      <c r="H17" s="16" t="n">
-        <v>2246.1</v>
-      </c>
-      <c r="I17" s="18">
-        <f>I8-I15+I12+I16</f>
-        <v/>
-      </c>
-      <c r="J17" s="18">
-        <f>J8-J15+J12+J16</f>
-        <v/>
-      </c>
-      <c r="K17" s="18">
-        <f>K8-K15+K12+K16</f>
-        <v/>
-      </c>
-      <c r="L17" s="18">
-        <f>L8-L15+L12+L16</f>
-        <v/>
-      </c>
-      <c r="M17" s="18">
-        <f>M8-M15+M12+M16</f>
-        <v/>
-      </c>
-      <c r="N17" s="18">
-        <f>N8-N15+N12+N16</f>
-        <v/>
-      </c>
-      <c r="O17" s="18">
-        <f>O8-O15+O12+O16</f>
-        <v/>
-      </c>
-      <c r="P17" s="18">
-        <f>P8-P15+P12+P16</f>
-        <v/>
-      </c>
-      <c r="Q17" s="18">
-        <f>Q8-Q15+Q12+Q16</f>
-        <v/>
-      </c>
-      <c r="R17" s="18">
-        <f>R8-R15+R12+R16</f>
+      <c r="C17" s="15" t="n">
+        <v>-124</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>-147.2</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>-71.59999999999999</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>-747.2</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>-1069.5</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <v>812.8999999999999</v>
+      </c>
+      <c r="I17" s="16">
+        <f>I10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="J17" s="16">
+        <f>J10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="K17" s="16">
+        <f>K10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="L17" s="16">
+        <f>L10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="M17" s="16">
+        <f>M10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="N17" s="16">
+        <f>N10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="O17" s="16">
+        <f>O10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="P17" s="16">
+        <f>P10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="Q17" s="16">
+        <f>Q10*in_other_operating_cash_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="R17" s="16">
+        <f>R10*in_other_operating_cash_share_of_capex</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Debt raised, net (actuals: change in the reported balance)</t>
+          <t>Cash from operations</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2375,69 +2405,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C18" s="16" t="n">
-        <v>0.1000000000000005</v>
-      </c>
-      <c r="D18" s="16" t="n">
-        <v>980</v>
-      </c>
-      <c r="E18" s="16" t="n">
-        <v>3120.6</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <v>20.89999999999964</v>
-      </c>
-      <c r="G18" s="16" t="n">
-        <v>4322.7</v>
-      </c>
-      <c r="H18" s="16" t="n">
-        <v>95.30000000000109</v>
+      <c r="C18" s="15" t="n">
+        <v>-184.1</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>-167.9</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>-80.59999999999999</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>834.3</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>2258</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>2246.1</v>
       </c>
       <c r="I18" s="17">
-        <f>I9*in_debt_share_of_capex</f>
+        <f>I9-I16+I13+I17</f>
         <v/>
       </c>
       <c r="J18" s="17">
-        <f>J9*in_debt_share_of_capex</f>
+        <f>J9-J16+J13+J17</f>
         <v/>
       </c>
       <c r="K18" s="17">
-        <f>K9*in_debt_share_of_capex</f>
+        <f>K9-K16+K13+K17</f>
         <v/>
       </c>
       <c r="L18" s="17">
-        <f>L9*in_debt_share_of_capex</f>
+        <f>L9-L16+L13+L17</f>
         <v/>
       </c>
       <c r="M18" s="17">
-        <f>M9*in_debt_share_of_capex</f>
+        <f>M9-M16+M13+M17</f>
         <v/>
       </c>
       <c r="N18" s="17">
-        <f>N9*in_debt_share_of_capex</f>
+        <f>N9-N16+N13+N17</f>
         <v/>
       </c>
       <c r="O18" s="17">
-        <f>O9*in_debt_share_of_capex</f>
+        <f>O9-O16+O13+O17</f>
         <v/>
       </c>
       <c r="P18" s="17">
-        <f>P9*in_debt_share_of_capex</f>
+        <f>P9-P16+P13+P17</f>
         <v/>
       </c>
       <c r="Q18" s="17">
-        <f>Q9*in_debt_share_of_capex</f>
+        <f>Q9-Q16+Q13+Q17</f>
         <v/>
       </c>
       <c r="R18" s="17">
-        <f>R9*in_debt_share_of_capex</f>
+        <f>R9-R16+R13+R17</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Debt, end of quarter</t>
+          <t>Debt raised, net (actuals: change in the reported balance)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2445,69 +2475,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C19" s="16" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="D19" s="16" t="n">
-        <v>986.2</v>
-      </c>
-      <c r="E19" s="16" t="n">
-        <v>4106.8</v>
-      </c>
-      <c r="F19" s="16" t="n">
-        <v>4127.7</v>
-      </c>
-      <c r="G19" s="16" t="n">
-        <v>8450.4</v>
-      </c>
-      <c r="H19" s="16" t="n">
-        <v>8545.700000000001</v>
-      </c>
-      <c r="I19" s="18">
-        <f>H19+I18</f>
-        <v/>
-      </c>
-      <c r="J19" s="18">
-        <f>I19+J18</f>
-        <v/>
-      </c>
-      <c r="K19" s="18">
-        <f>J19+K18</f>
-        <v/>
-      </c>
-      <c r="L19" s="18">
-        <f>K19+L18</f>
-        <v/>
-      </c>
-      <c r="M19" s="18">
-        <f>L19+M18</f>
-        <v/>
-      </c>
-      <c r="N19" s="18">
-        <f>M19+N18</f>
-        <v/>
-      </c>
-      <c r="O19" s="18">
-        <f>N19+O18</f>
-        <v/>
-      </c>
-      <c r="P19" s="18">
-        <f>O19+P18</f>
-        <v/>
-      </c>
-      <c r="Q19" s="18">
-        <f>P19+Q18</f>
-        <v/>
-      </c>
-      <c r="R19" s="18">
-        <f>Q19+R18</f>
+      <c r="C19" s="15" t="n">
+        <v>0.1000000000000005</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>980</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>3120.6</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>20.89999999999964</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>4322.7</v>
+      </c>
+      <c r="H19" s="15" t="n">
+        <v>95.30000000000109</v>
+      </c>
+      <c r="I19" s="16">
+        <f>I10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>J10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="K19" s="16">
+        <f>K10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="L19" s="16">
+        <f>L10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="M19" s="16">
+        <f>M10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="N19" s="16">
+        <f>N10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="O19" s="16">
+        <f>O10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="P19" s="16">
+        <f>P10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="Q19" s="16">
+        <f>Q10*in_debt_share_of_capex</f>
+        <v/>
+      </c>
+      <c r="R19" s="16">
+        <f>R10*in_debt_share_of_capex</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Equity raised and other investing and financing (plug to reported cash)</t>
+          <t>Debt, end of quarter</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2515,59 +2545,69 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C20" s="16" t="n">
-        <v>-274.6999999999999</v>
-      </c>
-      <c r="D20" s="16" t="n">
-        <v>-69.20000000000005</v>
-      </c>
-      <c r="E20" s="16" t="n">
-        <v>1031</v>
-      </c>
-      <c r="F20" s="16" t="n">
-        <v>84.10000000000014</v>
-      </c>
-      <c r="G20" s="16" t="n">
-        <v>1512.3</v>
-      </c>
-      <c r="H20" s="16" t="n">
-        <v>2059.899999999998</v>
-      </c>
-      <c r="I20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="16" t="n">
-        <v>0</v>
+      <c r="C20" s="15" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>986.2</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>4106.8</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>4127.7</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>8450.4</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v>8545.700000000001</v>
+      </c>
+      <c r="I20" s="17">
+        <f>H20+I19</f>
+        <v/>
+      </c>
+      <c r="J20" s="17">
+        <f>I20+J19</f>
+        <v/>
+      </c>
+      <c r="K20" s="17">
+        <f>J20+K19</f>
+        <v/>
+      </c>
+      <c r="L20" s="17">
+        <f>K20+L19</f>
+        <v/>
+      </c>
+      <c r="M20" s="17">
+        <f>L20+M19</f>
+        <v/>
+      </c>
+      <c r="N20" s="17">
+        <f>M20+N19</f>
+        <v/>
+      </c>
+      <c r="O20" s="17">
+        <f>N20+O19</f>
+        <v/>
+      </c>
+      <c r="P20" s="17">
+        <f>O20+P19</f>
+        <v/>
+      </c>
+      <c r="Q20" s="17">
+        <f>P20+Q19</f>
+        <v/>
+      </c>
+      <c r="R20" s="17">
+        <f>Q20+R19</f>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>External funding required to hold minimum cash (equity-like, no interest)</t>
+          <t>Equity raised and other investing and financing (plug to reported cash)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2575,132 +2615,192 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C21" s="16" t="n">
+      <c r="C21" s="15" t="n">
+        <v>-274.6999999999999</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>-69.20000000000005</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>1031</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>84.10000000000014</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>1512.3</v>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v>2059.899999999998</v>
+      </c>
+      <c r="I21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D21" s="16" t="n">
+      <c r="J21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="16" t="n">
+      <c r="K21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="16" t="n">
+      <c r="L21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="16" t="n">
+      <c r="M21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="16" t="n">
+      <c r="N21" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(H22+I17-I9+I18+I20))</f>
-        <v/>
-      </c>
-      <c r="J21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(I22+J17-J9+J18+J20))</f>
-        <v/>
-      </c>
-      <c r="K21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(J22+K17-K9+K18+K20))</f>
-        <v/>
-      </c>
-      <c r="L21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(K22+L17-L9+L18+L20))</f>
-        <v/>
-      </c>
-      <c r="M21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(L22+M17-M9+M18+M20))</f>
-        <v/>
-      </c>
-      <c r="N21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(M22+N17-N9+N18+N20))</f>
-        <v/>
-      </c>
-      <c r="O21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(N22+O17-O9+O18+O20))</f>
-        <v/>
-      </c>
-      <c r="P21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(O22+P17-P9+P18+P20))</f>
-        <v/>
-      </c>
-      <c r="Q21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(P22+Q17-Q9+Q18+Q20))</f>
-        <v/>
-      </c>
-      <c r="R21" s="17">
-        <f>MAX(0,in_minimum_cash_usd_bn*1000-(Q22+R17-R9+R18+R20))</f>
-        <v/>
+      <c r="O21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>External funding required to hold minimum cash (equity-like, no interest)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(H23+I18-I10+I19+I21))</f>
+        <v/>
+      </c>
+      <c r="J22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(I23+J18-J10+J19+J21))</f>
+        <v/>
+      </c>
+      <c r="K22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(J23+K18-K10+K19+K21))</f>
+        <v/>
+      </c>
+      <c r="L22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(K23+L18-L10+L19+L21))</f>
+        <v/>
+      </c>
+      <c r="M22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(L23+M18-M10+M19+M21))</f>
+        <v/>
+      </c>
+      <c r="N22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(M23+N18-N10+N19+N21))</f>
+        <v/>
+      </c>
+      <c r="O22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(N23+O18-O10+O19+O21))</f>
+        <v/>
+      </c>
+      <c r="P22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(O23+P18-P10+P19+P21))</f>
+        <v/>
+      </c>
+      <c r="Q22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(P23+Q18-Q10+Q19+Q21))</f>
+        <v/>
+      </c>
+      <c r="R22" s="16">
+        <f>MAX(0,in_minimum_cash_usd_bn*1000-(Q23+R18-R10+R19+R21))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Cash and cash equivalents, end of quarter</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>USD m</t>
         </is>
       </c>
-      <c r="C22" s="16" t="n">
+      <c r="C23" s="15" t="n">
         <v>1447</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D23" s="15" t="n">
         <v>1679.3</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E23" s="15" t="n">
         <v>4794.8</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="F23" s="15" t="n">
         <v>3678.1</v>
       </c>
-      <c r="G22" s="16" t="n">
+      <c r="G23" s="15" t="n">
         <v>9298.200000000001</v>
       </c>
-      <c r="H22" s="16" t="n">
+      <c r="H23" s="15" t="n">
         <v>8042.1</v>
       </c>
-      <c r="I22" s="18">
-        <f>H22+I17-I9+I18+I20+I21</f>
-        <v/>
-      </c>
-      <c r="J22" s="18">
-        <f>I22+J17-J9+J18+J20+J21</f>
-        <v/>
-      </c>
-      <c r="K22" s="18">
-        <f>J22+K17-K9+K18+K20+K21</f>
-        <v/>
-      </c>
-      <c r="L22" s="18">
-        <f>K22+L17-L9+L18+L20+L21</f>
-        <v/>
-      </c>
-      <c r="M22" s="18">
-        <f>L22+M17-M9+M18+M20+M21</f>
-        <v/>
-      </c>
-      <c r="N22" s="18">
-        <f>M22+N17-N9+N18+N20+N21</f>
-        <v/>
-      </c>
-      <c r="O22" s="18">
-        <f>N22+O17-O9+O18+O20+O21</f>
-        <v/>
-      </c>
-      <c r="P22" s="18">
-        <f>O22+P17-P9+P18+P20+P21</f>
-        <v/>
-      </c>
-      <c r="Q22" s="18">
-        <f>P22+Q17-Q9+Q18+Q20+Q21</f>
-        <v/>
-      </c>
-      <c r="R22" s="18">
-        <f>Q22+R17-R9+R18+R20+R21</f>
+      <c r="I23" s="17">
+        <f>H23+I18-I10+I19+I21+I22</f>
+        <v/>
+      </c>
+      <c r="J23" s="17">
+        <f>I23+J18-J10+J19+J21+J22</f>
+        <v/>
+      </c>
+      <c r="K23" s="17">
+        <f>J23+K18-K10+K19+K21+K22</f>
+        <v/>
+      </c>
+      <c r="L23" s="17">
+        <f>K23+L18-L10+L19+L21+L22</f>
+        <v/>
+      </c>
+      <c r="M23" s="17">
+        <f>L23+M18-M10+M19+M21+M22</f>
+        <v/>
+      </c>
+      <c r="N23" s="17">
+        <f>M23+N18-N10+N19+N21+N22</f>
+        <v/>
+      </c>
+      <c r="O23" s="17">
+        <f>N23+O18-O10+O19+O21+O22</f>
+        <v/>
+      </c>
+      <c r="P23" s="17">
+        <f>O23+P18-P10+P19+P21+P22</f>
+        <v/>
+      </c>
+      <c r="Q23" s="17">
+        <f>P23+Q18-Q10+Q19+Q21+Q22</f>
+        <v/>
+      </c>
+      <c r="R23" s="17">
+        <f>Q23+R18-R10+R19+R21+R22</f>
         <v/>
       </c>
     </row>
@@ -2841,67 +2941,67 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="18" t="n">
         <v>3.850877192982455</v>
       </c>
-      <c r="D2" s="20">
-        <f>Drivers!D7/Drivers!C7-1</f>
-        <v/>
-      </c>
-      <c r="E2" s="20">
-        <f>Drivers!E7/Drivers!D7-1</f>
-        <v/>
-      </c>
-      <c r="F2" s="20">
-        <f>Drivers!F7/Drivers!E7-1</f>
-        <v/>
-      </c>
-      <c r="G2" s="20">
-        <f>Drivers!G7/Drivers!F7-1</f>
-        <v/>
-      </c>
-      <c r="H2" s="20">
-        <f>Drivers!H7/Drivers!G7-1</f>
-        <v/>
-      </c>
-      <c r="I2" s="20">
-        <f>Drivers!I7/Drivers!H7-1</f>
-        <v/>
-      </c>
-      <c r="J2" s="20">
-        <f>Drivers!J7/Drivers!I7-1</f>
-        <v/>
-      </c>
-      <c r="K2" s="20">
-        <f>Drivers!K7/Drivers!J7-1</f>
-        <v/>
-      </c>
-      <c r="L2" s="20">
-        <f>Drivers!L7/Drivers!K7-1</f>
-        <v/>
-      </c>
-      <c r="M2" s="20">
-        <f>Drivers!M7/Drivers!L7-1</f>
-        <v/>
-      </c>
-      <c r="N2" s="20">
-        <f>Drivers!N7/Drivers!M7-1</f>
-        <v/>
-      </c>
-      <c r="O2" s="20">
-        <f>Drivers!O7/Drivers!N7-1</f>
-        <v/>
-      </c>
-      <c r="P2" s="20">
-        <f>Drivers!P7/Drivers!O7-1</f>
-        <v/>
-      </c>
-      <c r="Q2" s="20">
-        <f>Drivers!Q7/Drivers!P7-1</f>
-        <v/>
-      </c>
-      <c r="R2" s="20">
-        <f>Drivers!R7/Drivers!Q7-1</f>
+      <c r="D2" s="19">
+        <f>Drivers!D8/Drivers!C8-1</f>
+        <v/>
+      </c>
+      <c r="E2" s="19">
+        <f>Drivers!E8/Drivers!D8-1</f>
+        <v/>
+      </c>
+      <c r="F2" s="19">
+        <f>Drivers!F8/Drivers!E8-1</f>
+        <v/>
+      </c>
+      <c r="G2" s="19">
+        <f>Drivers!G8/Drivers!F8-1</f>
+        <v/>
+      </c>
+      <c r="H2" s="19">
+        <f>Drivers!H8/Drivers!G8-1</f>
+        <v/>
+      </c>
+      <c r="I2" s="19">
+        <f>Drivers!I8/Drivers!H8-1</f>
+        <v/>
+      </c>
+      <c r="J2" s="19">
+        <f>Drivers!J8/Drivers!I8-1</f>
+        <v/>
+      </c>
+      <c r="K2" s="19">
+        <f>Drivers!K8/Drivers!J8-1</f>
+        <v/>
+      </c>
+      <c r="L2" s="19">
+        <f>Drivers!L8/Drivers!K8-1</f>
+        <v/>
+      </c>
+      <c r="M2" s="19">
+        <f>Drivers!M8/Drivers!L8-1</f>
+        <v/>
+      </c>
+      <c r="N2" s="19">
+        <f>Drivers!N8/Drivers!M8-1</f>
+        <v/>
+      </c>
+      <c r="O2" s="19">
+        <f>Drivers!O8/Drivers!N8-1</f>
+        <v/>
+      </c>
+      <c r="P2" s="19">
+        <f>Drivers!P8/Drivers!O8-1</f>
+        <v/>
+      </c>
+      <c r="Q2" s="19">
+        <f>Drivers!Q8/Drivers!P8-1</f>
+        <v/>
+      </c>
+      <c r="R2" s="19">
+        <f>Drivers!R8/Drivers!Q8-1</f>
         <v/>
       </c>
     </row>
@@ -2916,68 +3016,68 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C3" s="20">
-        <f>Drivers!C8/Drivers!C7</f>
-        <v/>
-      </c>
-      <c r="D3" s="20">
-        <f>Drivers!D8/Drivers!D7</f>
-        <v/>
-      </c>
-      <c r="E3" s="20">
-        <f>Drivers!E8/Drivers!E7</f>
-        <v/>
-      </c>
-      <c r="F3" s="20">
-        <f>Drivers!F8/Drivers!F7</f>
-        <v/>
-      </c>
-      <c r="G3" s="20">
-        <f>Drivers!G8/Drivers!G7</f>
-        <v/>
-      </c>
-      <c r="H3" s="20">
-        <f>Drivers!H8/Drivers!H7</f>
-        <v/>
-      </c>
-      <c r="I3" s="20">
-        <f>Drivers!I8/Drivers!I7</f>
-        <v/>
-      </c>
-      <c r="J3" s="20">
-        <f>Drivers!J8/Drivers!J7</f>
-        <v/>
-      </c>
-      <c r="K3" s="20">
-        <f>Drivers!K8/Drivers!K7</f>
-        <v/>
-      </c>
-      <c r="L3" s="20">
-        <f>Drivers!L8/Drivers!L7</f>
-        <v/>
-      </c>
-      <c r="M3" s="20">
-        <f>Drivers!M8/Drivers!M7</f>
-        <v/>
-      </c>
-      <c r="N3" s="20">
-        <f>Drivers!N8/Drivers!N7</f>
-        <v/>
-      </c>
-      <c r="O3" s="20">
-        <f>Drivers!O8/Drivers!O7</f>
-        <v/>
-      </c>
-      <c r="P3" s="20">
-        <f>Drivers!P8/Drivers!P7</f>
-        <v/>
-      </c>
-      <c r="Q3" s="20">
-        <f>Drivers!Q8/Drivers!Q7</f>
-        <v/>
-      </c>
-      <c r="R3" s="20">
-        <f>Drivers!R8/Drivers!R7</f>
+      <c r="C3" s="19">
+        <f>Drivers!C9/Drivers!C8</f>
+        <v/>
+      </c>
+      <c r="D3" s="19">
+        <f>Drivers!D9/Drivers!D8</f>
+        <v/>
+      </c>
+      <c r="E3" s="19">
+        <f>Drivers!E9/Drivers!E8</f>
+        <v/>
+      </c>
+      <c r="F3" s="19">
+        <f>Drivers!F9/Drivers!F8</f>
+        <v/>
+      </c>
+      <c r="G3" s="19">
+        <f>Drivers!G9/Drivers!G8</f>
+        <v/>
+      </c>
+      <c r="H3" s="19">
+        <f>Drivers!H9/Drivers!H8</f>
+        <v/>
+      </c>
+      <c r="I3" s="19">
+        <f>Drivers!I9/Drivers!I8</f>
+        <v/>
+      </c>
+      <c r="J3" s="19">
+        <f>Drivers!J9/Drivers!J8</f>
+        <v/>
+      </c>
+      <c r="K3" s="19">
+        <f>Drivers!K9/Drivers!K8</f>
+        <v/>
+      </c>
+      <c r="L3" s="19">
+        <f>Drivers!L9/Drivers!L8</f>
+        <v/>
+      </c>
+      <c r="M3" s="19">
+        <f>Drivers!M9/Drivers!M8</f>
+        <v/>
+      </c>
+      <c r="N3" s="19">
+        <f>Drivers!N9/Drivers!N8</f>
+        <v/>
+      </c>
+      <c r="O3" s="19">
+        <f>Drivers!O9/Drivers!O8</f>
+        <v/>
+      </c>
+      <c r="P3" s="19">
+        <f>Drivers!P9/Drivers!P8</f>
+        <v/>
+      </c>
+      <c r="Q3" s="19">
+        <f>Drivers!Q9/Drivers!Q8</f>
+        <v/>
+      </c>
+      <c r="R3" s="19">
+        <f>Drivers!R9/Drivers!R8</f>
         <v/>
       </c>
     </row>
@@ -2992,68 +3092,68 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C4" s="20">
-        <f>Drivers!C6/Drivers!C7</f>
-        <v/>
-      </c>
-      <c r="D4" s="20">
-        <f>Drivers!D6/Drivers!D7</f>
-        <v/>
-      </c>
-      <c r="E4" s="20">
-        <f>Drivers!E6/Drivers!E7</f>
-        <v/>
-      </c>
-      <c r="F4" s="20">
-        <f>Drivers!F6/Drivers!F7</f>
-        <v/>
-      </c>
-      <c r="G4" s="20">
-        <f>Drivers!G6/Drivers!G7</f>
-        <v/>
-      </c>
-      <c r="H4" s="20">
-        <f>Drivers!H6/Drivers!H7</f>
-        <v/>
-      </c>
-      <c r="I4" s="20">
-        <f>Drivers!I6/Drivers!I7</f>
-        <v/>
-      </c>
-      <c r="J4" s="20">
-        <f>Drivers!J6/Drivers!J7</f>
-        <v/>
-      </c>
-      <c r="K4" s="20">
-        <f>Drivers!K6/Drivers!K7</f>
-        <v/>
-      </c>
-      <c r="L4" s="20">
-        <f>Drivers!L6/Drivers!L7</f>
-        <v/>
-      </c>
-      <c r="M4" s="20">
-        <f>Drivers!M6/Drivers!M7</f>
-        <v/>
-      </c>
-      <c r="N4" s="20">
-        <f>Drivers!N6/Drivers!N7</f>
-        <v/>
-      </c>
-      <c r="O4" s="20">
-        <f>Drivers!O6/Drivers!O7</f>
-        <v/>
-      </c>
-      <c r="P4" s="20">
-        <f>Drivers!P6/Drivers!P7</f>
-        <v/>
-      </c>
-      <c r="Q4" s="20">
-        <f>Drivers!Q6/Drivers!Q7</f>
-        <v/>
-      </c>
-      <c r="R4" s="20">
-        <f>Drivers!R6/Drivers!R7</f>
+      <c r="C4" s="19">
+        <f>Drivers!C7/Drivers!C8</f>
+        <v/>
+      </c>
+      <c r="D4" s="19">
+        <f>Drivers!D7/Drivers!D8</f>
+        <v/>
+      </c>
+      <c r="E4" s="19">
+        <f>Drivers!E7/Drivers!E8</f>
+        <v/>
+      </c>
+      <c r="F4" s="19">
+        <f>Drivers!F7/Drivers!F8</f>
+        <v/>
+      </c>
+      <c r="G4" s="19">
+        <f>Drivers!G7/Drivers!G8</f>
+        <v/>
+      </c>
+      <c r="H4" s="19">
+        <f>Drivers!H7/Drivers!H8</f>
+        <v/>
+      </c>
+      <c r="I4" s="19">
+        <f>Drivers!I7/Drivers!I8</f>
+        <v/>
+      </c>
+      <c r="J4" s="19">
+        <f>Drivers!J7/Drivers!J8</f>
+        <v/>
+      </c>
+      <c r="K4" s="19">
+        <f>Drivers!K7/Drivers!K8</f>
+        <v/>
+      </c>
+      <c r="L4" s="19">
+        <f>Drivers!L7/Drivers!L8</f>
+        <v/>
+      </c>
+      <c r="M4" s="19">
+        <f>Drivers!M7/Drivers!M8</f>
+        <v/>
+      </c>
+      <c r="N4" s="19">
+        <f>Drivers!N7/Drivers!N8</f>
+        <v/>
+      </c>
+      <c r="O4" s="19">
+        <f>Drivers!O7/Drivers!O8</f>
+        <v/>
+      </c>
+      <c r="P4" s="19">
+        <f>Drivers!P7/Drivers!P8</f>
+        <v/>
+      </c>
+      <c r="Q4" s="19">
+        <f>Drivers!Q7/Drivers!Q8</f>
+        <v/>
+      </c>
+      <c r="R4" s="19">
+        <f>Drivers!R7/Drivers!R8</f>
         <v/>
       </c>
     </row>
@@ -3069,64 +3169,64 @@
         </is>
       </c>
       <c r="C5" s="13" t="n"/>
-      <c r="D5" s="14">
-        <f>Drivers!D6/((Drivers!C5+Drivers!D5)/8)</f>
-        <v/>
-      </c>
-      <c r="E5" s="14">
-        <f>Drivers!E6/((Drivers!D5+Drivers!E5)/8)</f>
-        <v/>
-      </c>
-      <c r="F5" s="14">
-        <f>Drivers!F6/((Drivers!E5+Drivers!F5)/8)</f>
-        <v/>
-      </c>
-      <c r="G5" s="14">
-        <f>Drivers!G6/((Drivers!F5+Drivers!G5)/8)</f>
-        <v/>
-      </c>
-      <c r="H5" s="14">
-        <f>Drivers!H6/((Drivers!G5+Drivers!H5)/8)</f>
-        <v/>
-      </c>
-      <c r="I5" s="14">
-        <f>Drivers!I6/((Drivers!H5+Drivers!I5)/8)</f>
-        <v/>
-      </c>
-      <c r="J5" s="14">
-        <f>Drivers!J6/((Drivers!I5+Drivers!J5)/8)</f>
-        <v/>
-      </c>
-      <c r="K5" s="14">
-        <f>Drivers!K6/((Drivers!J5+Drivers!K5)/8)</f>
-        <v/>
-      </c>
-      <c r="L5" s="14">
-        <f>Drivers!L6/((Drivers!K5+Drivers!L5)/8)</f>
-        <v/>
-      </c>
-      <c r="M5" s="14">
-        <f>Drivers!M6/((Drivers!L5+Drivers!M5)/8)</f>
-        <v/>
-      </c>
-      <c r="N5" s="14">
-        <f>Drivers!N6/((Drivers!M5+Drivers!N5)/8)</f>
-        <v/>
-      </c>
-      <c r="O5" s="14">
-        <f>Drivers!O6/((Drivers!N5+Drivers!O5)/8)</f>
-        <v/>
-      </c>
-      <c r="P5" s="14">
-        <f>Drivers!P6/((Drivers!O5+Drivers!P5)/8)</f>
-        <v/>
-      </c>
-      <c r="Q5" s="14">
-        <f>Drivers!Q6/((Drivers!P5+Drivers!Q5)/8)</f>
-        <v/>
-      </c>
-      <c r="R5" s="14">
-        <f>Drivers!R6/((Drivers!Q5+Drivers!R5)/8)</f>
+      <c r="D5" s="20">
+        <f>Drivers!D7/((Drivers!C6+Drivers!D6)/8)</f>
+        <v/>
+      </c>
+      <c r="E5" s="20">
+        <f>Drivers!E7/((Drivers!D6+Drivers!E6)/8)</f>
+        <v/>
+      </c>
+      <c r="F5" s="20">
+        <f>Drivers!F7/((Drivers!E6+Drivers!F6)/8)</f>
+        <v/>
+      </c>
+      <c r="G5" s="20">
+        <f>Drivers!G7/((Drivers!F6+Drivers!G6)/8)</f>
+        <v/>
+      </c>
+      <c r="H5" s="20">
+        <f>Drivers!H7/((Drivers!G6+Drivers!H6)/8)</f>
+        <v/>
+      </c>
+      <c r="I5" s="20">
+        <f>Drivers!I7/((Drivers!H6+Drivers!I6)/8)</f>
+        <v/>
+      </c>
+      <c r="J5" s="20">
+        <f>Drivers!J7/((Drivers!I6+Drivers!J6)/8)</f>
+        <v/>
+      </c>
+      <c r="K5" s="20">
+        <f>Drivers!K7/((Drivers!J6+Drivers!K6)/8)</f>
+        <v/>
+      </c>
+      <c r="L5" s="20">
+        <f>Drivers!L7/((Drivers!K6+Drivers!L6)/8)</f>
+        <v/>
+      </c>
+      <c r="M5" s="20">
+        <f>Drivers!M7/((Drivers!L6+Drivers!M6)/8)</f>
+        <v/>
+      </c>
+      <c r="N5" s="20">
+        <f>Drivers!N7/((Drivers!M6+Drivers!N6)/8)</f>
+        <v/>
+      </c>
+      <c r="O5" s="20">
+        <f>Drivers!O7/((Drivers!N6+Drivers!O6)/8)</f>
+        <v/>
+      </c>
+      <c r="P5" s="20">
+        <f>Drivers!P7/((Drivers!O6+Drivers!P6)/8)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="20">
+        <f>Drivers!Q7/((Drivers!P6+Drivers!Q6)/8)</f>
+        <v/>
+      </c>
+      <c r="R5" s="20">
+        <f>Drivers!R7/((Drivers!Q6+Drivers!R6)/8)</f>
         <v/>
       </c>
     </row>
@@ -3141,68 +3241,68 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C6" s="17">
-        <f>Drivers!C5/Drivers!C2</f>
-        <v/>
-      </c>
-      <c r="D6" s="17">
-        <f>Drivers!D5/Drivers!D2</f>
-        <v/>
-      </c>
-      <c r="E6" s="17">
-        <f>Drivers!E5/Drivers!E2</f>
-        <v/>
-      </c>
-      <c r="F6" s="17">
-        <f>Drivers!F5/Drivers!F2</f>
-        <v/>
-      </c>
-      <c r="G6" s="17">
-        <f>Drivers!G5/Drivers!G2</f>
-        <v/>
-      </c>
-      <c r="H6" s="17">
-        <f>Drivers!H5/Drivers!H2</f>
-        <v/>
-      </c>
-      <c r="I6" s="17">
-        <f>Drivers!I5/Drivers!I2</f>
-        <v/>
-      </c>
-      <c r="J6" s="17">
-        <f>Drivers!J5/Drivers!J2</f>
-        <v/>
-      </c>
-      <c r="K6" s="17">
-        <f>Drivers!K5/Drivers!K2</f>
-        <v/>
-      </c>
-      <c r="L6" s="17">
-        <f>Drivers!L5/Drivers!L2</f>
-        <v/>
-      </c>
-      <c r="M6" s="17">
-        <f>Drivers!M5/Drivers!M2</f>
-        <v/>
-      </c>
-      <c r="N6" s="17">
-        <f>Drivers!N5/Drivers!N2</f>
-        <v/>
-      </c>
-      <c r="O6" s="17">
-        <f>Drivers!O5/Drivers!O2</f>
-        <v/>
-      </c>
-      <c r="P6" s="17">
-        <f>Drivers!P5/Drivers!P2</f>
-        <v/>
-      </c>
-      <c r="Q6" s="17">
-        <f>Drivers!Q5/Drivers!Q2</f>
-        <v/>
-      </c>
-      <c r="R6" s="17">
-        <f>Drivers!R5/Drivers!R2</f>
+      <c r="C6" s="16">
+        <f>Drivers!C6/Drivers!C3</f>
+        <v/>
+      </c>
+      <c r="D6" s="16">
+        <f>Drivers!D6/Drivers!D3</f>
+        <v/>
+      </c>
+      <c r="E6" s="16">
+        <f>Drivers!E6/Drivers!E3</f>
+        <v/>
+      </c>
+      <c r="F6" s="16">
+        <f>Drivers!F6/Drivers!F3</f>
+        <v/>
+      </c>
+      <c r="G6" s="16">
+        <f>Drivers!G6/Drivers!G3</f>
+        <v/>
+      </c>
+      <c r="H6" s="16">
+        <f>Drivers!H6/Drivers!H3</f>
+        <v/>
+      </c>
+      <c r="I6" s="16">
+        <f>Drivers!I6/Drivers!I3</f>
+        <v/>
+      </c>
+      <c r="J6" s="16">
+        <f>Drivers!J6/Drivers!J3</f>
+        <v/>
+      </c>
+      <c r="K6" s="16">
+        <f>Drivers!K6/Drivers!K3</f>
+        <v/>
+      </c>
+      <c r="L6" s="16">
+        <f>Drivers!L6/Drivers!L3</f>
+        <v/>
+      </c>
+      <c r="M6" s="16">
+        <f>Drivers!M6/Drivers!M3</f>
+        <v/>
+      </c>
+      <c r="N6" s="16">
+        <f>Drivers!N6/Drivers!N3</f>
+        <v/>
+      </c>
+      <c r="O6" s="16">
+        <f>Drivers!O6/Drivers!O3</f>
+        <v/>
+      </c>
+      <c r="P6" s="16">
+        <f>Drivers!P6/Drivers!P3</f>
+        <v/>
+      </c>
+      <c r="Q6" s="16">
+        <f>Drivers!Q6/Drivers!Q3</f>
+        <v/>
+      </c>
+      <c r="R6" s="16">
+        <f>Drivers!R6/Drivers!R3</f>
         <v/>
       </c>
     </row>
@@ -3217,67 +3317,67 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="K7" s="17">
+      <c r="K7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="L7" s="17">
+      <c r="L7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="M7" s="17">
+      <c r="M7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="N7" s="17">
+      <c r="N7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="P7" s="17">
+      <c r="P7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="Q7" s="17">
+      <c r="Q7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="R7" s="17">
+      <c r="R7" s="16">
         <f>in_arr_guidance_ye2026_low_usd_m</f>
         <v/>
       </c>
@@ -3293,67 +3393,67 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="G8" s="17">
+      <c r="G8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="H8" s="17">
+      <c r="H8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="I8" s="17">
+      <c r="I8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="J8" s="17">
+      <c r="J8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="K8" s="17">
+      <c r="K8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="L8" s="17">
+      <c r="L8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="M8" s="17">
+      <c r="M8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="N8" s="17">
+      <c r="N8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="O8" s="17">
+      <c r="O8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="P8" s="17">
+      <c r="P8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="Q8" s="17">
+      <c r="Q8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="R8" s="17">
+      <c r="R8" s="16">
         <f>in_arr_guidance_ye2026_high_usd_m</f>
         <v/>
       </c>
@@ -3369,67 +3469,67 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="I9" s="17">
+      <c r="I9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="J9" s="17">
+      <c r="J9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="K9" s="17">
+      <c r="K9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="L9" s="17">
+      <c r="L9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="M9" s="17">
+      <c r="M9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="N9" s="17">
+      <c r="N9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="O9" s="17">
+      <c r="O9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="P9" s="17">
+      <c r="P9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="Q9" s="17">
+      <c r="Q9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
-      <c r="R9" s="17">
+      <c r="R9" s="16">
         <f>in_revenue_guidance_2026_low_usd_m</f>
         <v/>
       </c>
@@ -3445,67 +3545,67 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="H10" s="17">
+      <c r="H10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="I10" s="17">
+      <c r="I10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="J10" s="17">
+      <c r="J10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="K10" s="17">
+      <c r="K10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="L10" s="17">
+      <c r="L10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="M10" s="17">
+      <c r="M10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="N10" s="17">
+      <c r="N10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="O10" s="17">
+      <c r="O10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="P10" s="17">
+      <c r="P10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="Q10" s="17">
+      <c r="Q10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
-      <c r="R10" s="17">
+      <c r="R10" s="16">
         <f>in_revenue_guidance_2026_high_usd_m</f>
         <v/>
       </c>
@@ -3521,50 +3621,50 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="17">
-        <f>Drivers!I8*4/Drivers!I4</f>
-        <v/>
-      </c>
-      <c r="J11" s="17">
-        <f>Drivers!J8*4/Drivers!J4</f>
-        <v/>
-      </c>
-      <c r="K11" s="17">
-        <f>Drivers!K8*4/Drivers!K4</f>
-        <v/>
-      </c>
-      <c r="L11" s="17">
-        <f>Drivers!L8*4/Drivers!L4</f>
-        <v/>
-      </c>
-      <c r="M11" s="17">
-        <f>Drivers!M8*4/Drivers!M4</f>
-        <v/>
-      </c>
-      <c r="N11" s="17">
-        <f>Drivers!N8*4/Drivers!N4</f>
-        <v/>
-      </c>
-      <c r="O11" s="17">
-        <f>Drivers!O8*4/Drivers!O4</f>
-        <v/>
-      </c>
-      <c r="P11" s="17">
-        <f>Drivers!P8*4/Drivers!P4</f>
-        <v/>
-      </c>
-      <c r="Q11" s="17">
-        <f>Drivers!Q8*4/Drivers!Q4</f>
-        <v/>
-      </c>
-      <c r="R11" s="17">
-        <f>Drivers!R8*4/Drivers!R4</f>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="16">
+        <f>Drivers!I9*4/Drivers!I5</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>Drivers!J9*4/Drivers!J5</f>
+        <v/>
+      </c>
+      <c r="K11" s="16">
+        <f>Drivers!K9*4/Drivers!K5</f>
+        <v/>
+      </c>
+      <c r="L11" s="16">
+        <f>Drivers!L9*4/Drivers!L5</f>
+        <v/>
+      </c>
+      <c r="M11" s="16">
+        <f>Drivers!M9*4/Drivers!M5</f>
+        <v/>
+      </c>
+      <c r="N11" s="16">
+        <f>Drivers!N9*4/Drivers!N5</f>
+        <v/>
+      </c>
+      <c r="O11" s="16">
+        <f>Drivers!O9*4/Drivers!O5</f>
+        <v/>
+      </c>
+      <c r="P11" s="16">
+        <f>Drivers!P9*4/Drivers!P5</f>
+        <v/>
+      </c>
+      <c r="Q11" s="16">
+        <f>Drivers!Q9*4/Drivers!Q5</f>
+        <v/>
+      </c>
+      <c r="R11" s="16">
+        <f>Drivers!R9*4/Drivers!R5</f>
         <v/>
       </c>
     </row>
@@ -3585,43 +3685,43 @@
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
       <c r="H12" s="13" t="n"/>
-      <c r="I12" s="14">
+      <c r="I12" s="20">
         <f>in_capex_per_mw_usd_m/I11</f>
         <v/>
       </c>
-      <c r="J12" s="14">
+      <c r="J12" s="20">
         <f>in_capex_per_mw_usd_m/J11</f>
         <v/>
       </c>
-      <c r="K12" s="14">
+      <c r="K12" s="20">
         <f>in_capex_per_mw_usd_m/K11</f>
         <v/>
       </c>
-      <c r="L12" s="14">
+      <c r="L12" s="20">
         <f>in_capex_per_mw_usd_m/L11</f>
         <v/>
       </c>
-      <c r="M12" s="14">
+      <c r="M12" s="20">
         <f>in_capex_per_mw_usd_m/M11</f>
         <v/>
       </c>
-      <c r="N12" s="14">
+      <c r="N12" s="20">
         <f>in_capex_per_mw_usd_m/N11</f>
         <v/>
       </c>
-      <c r="O12" s="14">
+      <c r="O12" s="20">
         <f>in_capex_per_mw_usd_m/O11</f>
         <v/>
       </c>
-      <c r="P12" s="14">
+      <c r="P12" s="20">
         <f>in_capex_per_mw_usd_m/P11</f>
         <v/>
       </c>
-      <c r="Q12" s="14">
+      <c r="Q12" s="20">
         <f>in_capex_per_mw_usd_m/Q11</f>
         <v/>
       </c>
-      <c r="R12" s="14">
+      <c r="R12" s="20">
         <f>in_capex_per_mw_usd_m/R11</f>
         <v/>
       </c>
@@ -3643,43 +3743,43 @@
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n"/>
       <c r="H13" s="13" t="n"/>
-      <c r="I13" s="14">
+      <c r="I13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/I11</f>
         <v/>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/J11</f>
         <v/>
       </c>
-      <c r="K13" s="14">
+      <c r="K13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/K11</f>
         <v/>
       </c>
-      <c r="L13" s="14">
+      <c r="L13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/L11</f>
         <v/>
       </c>
-      <c r="M13" s="14">
+      <c r="M13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/M11</f>
         <v/>
       </c>
-      <c r="N13" s="14">
+      <c r="N13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/N11</f>
         <v/>
       </c>
-      <c r="O13" s="14">
+      <c r="O13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/O11</f>
         <v/>
       </c>
-      <c r="P13" s="14">
+      <c r="P13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/P11</f>
         <v/>
       </c>
-      <c r="Q13" s="14">
+      <c r="Q13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/Q11</f>
         <v/>
       </c>
-      <c r="R13" s="14">
+      <c r="R13" s="20">
         <f>in_capex_per_mw_usd_m*(1-in_prepayment_share_of_capex)/R11</f>
         <v/>
       </c>
@@ -3695,67 +3795,67 @@
           <t>years</t>
         </is>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="H14" s="14">
+      <c r="H14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="I14" s="14">
+      <c r="I14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="K14" s="14">
+      <c r="K14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="L14" s="14">
+      <c r="L14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="M14" s="14">
+      <c r="M14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="N14" s="14">
+      <c r="N14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="O14" s="14">
+      <c r="O14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="P14" s="14">
+      <c r="P14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="Q14" s="14">
+      <c r="Q14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
-      <c r="R14" s="14">
+      <c r="R14" s="20">
         <f>in_disclosed_payback_months/12</f>
         <v/>
       </c>
@@ -3771,62 +3871,62 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="18" t="n">
         <v>0.00459643316786174</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="18" t="n">
         <v>0.0005875440658049368</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="18" t="n">
         <v>-0.003976975405546834</v>
       </c>
-      <c r="F15" s="19" t="n">
+      <c r="F15" s="18" t="n">
         <v>0.7619163424124513</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="G15" s="18" t="n">
         <v>1.293218488414412</v>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H15" s="18" t="n">
         <v>0.2115812917594655</v>
       </c>
-      <c r="I15" s="20">
-        <f>Drivers!I10/Drivers!I9</f>
-        <v/>
-      </c>
-      <c r="J15" s="20">
-        <f>Drivers!J10/Drivers!J9</f>
-        <v/>
-      </c>
-      <c r="K15" s="20">
-        <f>Drivers!K10/Drivers!K9</f>
-        <v/>
-      </c>
-      <c r="L15" s="20">
-        <f>Drivers!L10/Drivers!L9</f>
-        <v/>
-      </c>
-      <c r="M15" s="20">
-        <f>Drivers!M10/Drivers!M9</f>
-        <v/>
-      </c>
-      <c r="N15" s="20">
-        <f>Drivers!N10/Drivers!N9</f>
-        <v/>
-      </c>
-      <c r="O15" s="20">
-        <f>Drivers!O10/Drivers!O9</f>
-        <v/>
-      </c>
-      <c r="P15" s="20">
-        <f>Drivers!P10/Drivers!P9</f>
-        <v/>
-      </c>
-      <c r="Q15" s="20">
-        <f>Drivers!Q10/Drivers!Q9</f>
-        <v/>
-      </c>
-      <c r="R15" s="20">
-        <f>Drivers!R10/Drivers!R9</f>
+      <c r="I15" s="19">
+        <f>Drivers!I11/Drivers!I10</f>
+        <v/>
+      </c>
+      <c r="J15" s="19">
+        <f>Drivers!J11/Drivers!J10</f>
+        <v/>
+      </c>
+      <c r="K15" s="19">
+        <f>Drivers!K11/Drivers!K10</f>
+        <v/>
+      </c>
+      <c r="L15" s="19">
+        <f>Drivers!L11/Drivers!L10</f>
+        <v/>
+      </c>
+      <c r="M15" s="19">
+        <f>Drivers!M11/Drivers!M10</f>
+        <v/>
+      </c>
+      <c r="N15" s="19">
+        <f>Drivers!N11/Drivers!N10</f>
+        <v/>
+      </c>
+      <c r="O15" s="19">
+        <f>Drivers!O11/Drivers!O10</f>
+        <v/>
+      </c>
+      <c r="P15" s="19">
+        <f>Drivers!P11/Drivers!P10</f>
+        <v/>
+      </c>
+      <c r="Q15" s="19">
+        <f>Drivers!Q11/Drivers!Q10</f>
+        <v/>
+      </c>
+      <c r="R15" s="19">
+        <f>Drivers!R11/Drivers!R10</f>
         <v/>
       </c>
     </row>
@@ -3841,68 +3941,68 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C16" s="17">
-        <f>Drivers!C17-Drivers!C9</f>
-        <v/>
-      </c>
-      <c r="D16" s="17">
-        <f>Drivers!D17-Drivers!D9</f>
-        <v/>
-      </c>
-      <c r="E16" s="17">
-        <f>Drivers!E17-Drivers!E9</f>
-        <v/>
-      </c>
-      <c r="F16" s="17">
-        <f>Drivers!F17-Drivers!F9</f>
-        <v/>
-      </c>
-      <c r="G16" s="17">
-        <f>Drivers!G17-Drivers!G9</f>
-        <v/>
-      </c>
-      <c r="H16" s="17">
-        <f>Drivers!H17-Drivers!H9</f>
-        <v/>
-      </c>
-      <c r="I16" s="17">
-        <f>Drivers!I17-Drivers!I9</f>
-        <v/>
-      </c>
-      <c r="J16" s="17">
-        <f>Drivers!J17-Drivers!J9</f>
-        <v/>
-      </c>
-      <c r="K16" s="17">
-        <f>Drivers!K17-Drivers!K9</f>
-        <v/>
-      </c>
-      <c r="L16" s="17">
-        <f>Drivers!L17-Drivers!L9</f>
-        <v/>
-      </c>
-      <c r="M16" s="17">
-        <f>Drivers!M17-Drivers!M9</f>
-        <v/>
-      </c>
-      <c r="N16" s="17">
-        <f>Drivers!N17-Drivers!N9</f>
-        <v/>
-      </c>
-      <c r="O16" s="17">
-        <f>Drivers!O17-Drivers!O9</f>
-        <v/>
-      </c>
-      <c r="P16" s="17">
-        <f>Drivers!P17-Drivers!P9</f>
-        <v/>
-      </c>
-      <c r="Q16" s="17">
-        <f>Drivers!Q17-Drivers!Q9</f>
-        <v/>
-      </c>
-      <c r="R16" s="17">
-        <f>Drivers!R17-Drivers!R9</f>
+      <c r="C16" s="16">
+        <f>Drivers!C18-Drivers!C10</f>
+        <v/>
+      </c>
+      <c r="D16" s="16">
+        <f>Drivers!D18-Drivers!D10</f>
+        <v/>
+      </c>
+      <c r="E16" s="16">
+        <f>Drivers!E18-Drivers!E10</f>
+        <v/>
+      </c>
+      <c r="F16" s="16">
+        <f>Drivers!F18-Drivers!F10</f>
+        <v/>
+      </c>
+      <c r="G16" s="16">
+        <f>Drivers!G18-Drivers!G10</f>
+        <v/>
+      </c>
+      <c r="H16" s="16">
+        <f>Drivers!H18-Drivers!H10</f>
+        <v/>
+      </c>
+      <c r="I16" s="16">
+        <f>Drivers!I18-Drivers!I10</f>
+        <v/>
+      </c>
+      <c r="J16" s="16">
+        <f>Drivers!J18-Drivers!J10</f>
+        <v/>
+      </c>
+      <c r="K16" s="16">
+        <f>Drivers!K18-Drivers!K10</f>
+        <v/>
+      </c>
+      <c r="L16" s="16">
+        <f>Drivers!L18-Drivers!L10</f>
+        <v/>
+      </c>
+      <c r="M16" s="16">
+        <f>Drivers!M18-Drivers!M10</f>
+        <v/>
+      </c>
+      <c r="N16" s="16">
+        <f>Drivers!N18-Drivers!N10</f>
+        <v/>
+      </c>
+      <c r="O16" s="16">
+        <f>Drivers!O18-Drivers!O10</f>
+        <v/>
+      </c>
+      <c r="P16" s="16">
+        <f>Drivers!P18-Drivers!P10</f>
+        <v/>
+      </c>
+      <c r="Q16" s="16">
+        <f>Drivers!Q18-Drivers!Q10</f>
+        <v/>
+      </c>
+      <c r="R16" s="16">
+        <f>Drivers!R18-Drivers!R10</f>
         <v/>
       </c>
     </row>
@@ -3917,68 +4017,68 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C17" s="17">
-        <f>Drivers!C19-Drivers!C22</f>
-        <v/>
-      </c>
-      <c r="D17" s="17">
-        <f>Drivers!D19-Drivers!D22</f>
-        <v/>
-      </c>
-      <c r="E17" s="17">
-        <f>Drivers!E19-Drivers!E22</f>
-        <v/>
-      </c>
-      <c r="F17" s="17">
-        <f>Drivers!F19-Drivers!F22</f>
-        <v/>
-      </c>
-      <c r="G17" s="17">
-        <f>Drivers!G19-Drivers!G22</f>
-        <v/>
-      </c>
-      <c r="H17" s="17">
-        <f>Drivers!H19-Drivers!H22</f>
-        <v/>
-      </c>
-      <c r="I17" s="17">
-        <f>Drivers!I19-Drivers!I22</f>
-        <v/>
-      </c>
-      <c r="J17" s="17">
-        <f>Drivers!J19-Drivers!J22</f>
-        <v/>
-      </c>
-      <c r="K17" s="17">
-        <f>Drivers!K19-Drivers!K22</f>
-        <v/>
-      </c>
-      <c r="L17" s="17">
-        <f>Drivers!L19-Drivers!L22</f>
-        <v/>
-      </c>
-      <c r="M17" s="17">
-        <f>Drivers!M19-Drivers!M22</f>
-        <v/>
-      </c>
-      <c r="N17" s="17">
-        <f>Drivers!N19-Drivers!N22</f>
-        <v/>
-      </c>
-      <c r="O17" s="17">
-        <f>Drivers!O19-Drivers!O22</f>
-        <v/>
-      </c>
-      <c r="P17" s="17">
-        <f>Drivers!P19-Drivers!P22</f>
-        <v/>
-      </c>
-      <c r="Q17" s="17">
-        <f>Drivers!Q19-Drivers!Q22</f>
-        <v/>
-      </c>
-      <c r="R17" s="17">
-        <f>Drivers!R19-Drivers!R22</f>
+      <c r="C17" s="16">
+        <f>Drivers!C20-Drivers!C23</f>
+        <v/>
+      </c>
+      <c r="D17" s="16">
+        <f>Drivers!D20-Drivers!D23</f>
+        <v/>
+      </c>
+      <c r="E17" s="16">
+        <f>Drivers!E20-Drivers!E23</f>
+        <v/>
+      </c>
+      <c r="F17" s="16">
+        <f>Drivers!F20-Drivers!F23</f>
+        <v/>
+      </c>
+      <c r="G17" s="16">
+        <f>Drivers!G20-Drivers!G23</f>
+        <v/>
+      </c>
+      <c r="H17" s="16">
+        <f>Drivers!H20-Drivers!H23</f>
+        <v/>
+      </c>
+      <c r="I17" s="16">
+        <f>Drivers!I20-Drivers!I23</f>
+        <v/>
+      </c>
+      <c r="J17" s="16">
+        <f>Drivers!J20-Drivers!J23</f>
+        <v/>
+      </c>
+      <c r="K17" s="16">
+        <f>Drivers!K20-Drivers!K23</f>
+        <v/>
+      </c>
+      <c r="L17" s="16">
+        <f>Drivers!L20-Drivers!L23</f>
+        <v/>
+      </c>
+      <c r="M17" s="16">
+        <f>Drivers!M20-Drivers!M23</f>
+        <v/>
+      </c>
+      <c r="N17" s="16">
+        <f>Drivers!N20-Drivers!N23</f>
+        <v/>
+      </c>
+      <c r="O17" s="16">
+        <f>Drivers!O20-Drivers!O23</f>
+        <v/>
+      </c>
+      <c r="P17" s="16">
+        <f>Drivers!P20-Drivers!P23</f>
+        <v/>
+      </c>
+      <c r="Q17" s="16">
+        <f>Drivers!Q20-Drivers!Q23</f>
+        <v/>
+      </c>
+      <c r="R17" s="16">
+        <f>Drivers!R20-Drivers!R23</f>
         <v/>
       </c>
     </row>
@@ -3993,68 +4093,68 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C18" s="14">
-        <f>C17/(Drivers!C8*4)</f>
-        <v/>
-      </c>
-      <c r="D18" s="14">
-        <f>D17/(Drivers!D8*4)</f>
-        <v/>
-      </c>
-      <c r="E18" s="14">
-        <f>E17/(Drivers!E8*4)</f>
-        <v/>
-      </c>
-      <c r="F18" s="14">
-        <f>F17/(Drivers!F8*4)</f>
-        <v/>
-      </c>
-      <c r="G18" s="14">
-        <f>G17/(Drivers!G8*4)</f>
-        <v/>
-      </c>
-      <c r="H18" s="14">
-        <f>H17/(Drivers!H8*4)</f>
-        <v/>
-      </c>
-      <c r="I18" s="14">
-        <f>I17/(Drivers!I8*4)</f>
-        <v/>
-      </c>
-      <c r="J18" s="14">
-        <f>J17/(Drivers!J8*4)</f>
-        <v/>
-      </c>
-      <c r="K18" s="14">
-        <f>K17/(Drivers!K8*4)</f>
-        <v/>
-      </c>
-      <c r="L18" s="14">
-        <f>L17/(Drivers!L8*4)</f>
-        <v/>
-      </c>
-      <c r="M18" s="14">
-        <f>M17/(Drivers!M8*4)</f>
-        <v/>
-      </c>
-      <c r="N18" s="14">
-        <f>N17/(Drivers!N8*4)</f>
-        <v/>
-      </c>
-      <c r="O18" s="14">
-        <f>O17/(Drivers!O8*4)</f>
-        <v/>
-      </c>
-      <c r="P18" s="14">
-        <f>P17/(Drivers!P8*4)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="14">
-        <f>Q17/(Drivers!Q8*4)</f>
-        <v/>
-      </c>
-      <c r="R18" s="14">
-        <f>R17/(Drivers!R8*4)</f>
+      <c r="C18" s="20">
+        <f>C17/(Drivers!C9*4)</f>
+        <v/>
+      </c>
+      <c r="D18" s="20">
+        <f>D17/(Drivers!D9*4)</f>
+        <v/>
+      </c>
+      <c r="E18" s="20">
+        <f>E17/(Drivers!E9*4)</f>
+        <v/>
+      </c>
+      <c r="F18" s="20">
+        <f>F17/(Drivers!F9*4)</f>
+        <v/>
+      </c>
+      <c r="G18" s="20">
+        <f>G17/(Drivers!G9*4)</f>
+        <v/>
+      </c>
+      <c r="H18" s="20">
+        <f>H17/(Drivers!H9*4)</f>
+        <v/>
+      </c>
+      <c r="I18" s="20">
+        <f>I17/(Drivers!I9*4)</f>
+        <v/>
+      </c>
+      <c r="J18" s="20">
+        <f>J17/(Drivers!J9*4)</f>
+        <v/>
+      </c>
+      <c r="K18" s="20">
+        <f>K17/(Drivers!K9*4)</f>
+        <v/>
+      </c>
+      <c r="L18" s="20">
+        <f>L17/(Drivers!L9*4)</f>
+        <v/>
+      </c>
+      <c r="M18" s="20">
+        <f>M17/(Drivers!M9*4)</f>
+        <v/>
+      </c>
+      <c r="N18" s="20">
+        <f>N17/(Drivers!N9*4)</f>
+        <v/>
+      </c>
+      <c r="O18" s="20">
+        <f>O17/(Drivers!O9*4)</f>
+        <v/>
+      </c>
+      <c r="P18" s="20">
+        <f>P17/(Drivers!P9*4)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="20">
+        <f>Q17/(Drivers!Q9*4)</f>
+        <v/>
+      </c>
+      <c r="R18" s="20">
+        <f>R17/(Drivers!R9*4)</f>
         <v/>
       </c>
     </row>
@@ -4069,67 +4169,67 @@
           <t>USD m</t>
         </is>
       </c>
-      <c r="C19" s="16" t="n">
+      <c r="C19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="17">
-        <f>C19+Drivers!D21</f>
-        <v/>
-      </c>
-      <c r="E19" s="17">
-        <f>D19+Drivers!E21</f>
-        <v/>
-      </c>
-      <c r="F19" s="17">
-        <f>E19+Drivers!F21</f>
-        <v/>
-      </c>
-      <c r="G19" s="17">
-        <f>F19+Drivers!G21</f>
-        <v/>
-      </c>
-      <c r="H19" s="17">
-        <f>G19+Drivers!H21</f>
-        <v/>
-      </c>
-      <c r="I19" s="17">
-        <f>H19+Drivers!I21</f>
-        <v/>
-      </c>
-      <c r="J19" s="17">
-        <f>I19+Drivers!J21</f>
-        <v/>
-      </c>
-      <c r="K19" s="17">
-        <f>J19+Drivers!K21</f>
-        <v/>
-      </c>
-      <c r="L19" s="17">
-        <f>K19+Drivers!L21</f>
-        <v/>
-      </c>
-      <c r="M19" s="17">
-        <f>L19+Drivers!M21</f>
-        <v/>
-      </c>
-      <c r="N19" s="17">
-        <f>M19+Drivers!N21</f>
-        <v/>
-      </c>
-      <c r="O19" s="17">
-        <f>N19+Drivers!O21</f>
-        <v/>
-      </c>
-      <c r="P19" s="17">
-        <f>O19+Drivers!P21</f>
-        <v/>
-      </c>
-      <c r="Q19" s="17">
-        <f>P19+Drivers!Q21</f>
-        <v/>
-      </c>
-      <c r="R19" s="17">
-        <f>Q19+Drivers!R21</f>
+      <c r="D19" s="16">
+        <f>C19+Drivers!D22</f>
+        <v/>
+      </c>
+      <c r="E19" s="16">
+        <f>D19+Drivers!E22</f>
+        <v/>
+      </c>
+      <c r="F19" s="16">
+        <f>E19+Drivers!F22</f>
+        <v/>
+      </c>
+      <c r="G19" s="16">
+        <f>F19+Drivers!G22</f>
+        <v/>
+      </c>
+      <c r="H19" s="16">
+        <f>G19+Drivers!H22</f>
+        <v/>
+      </c>
+      <c r="I19" s="16">
+        <f>H19+Drivers!I22</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>I19+Drivers!J22</f>
+        <v/>
+      </c>
+      <c r="K19" s="16">
+        <f>J19+Drivers!K22</f>
+        <v/>
+      </c>
+      <c r="L19" s="16">
+        <f>K19+Drivers!L22</f>
+        <v/>
+      </c>
+      <c r="M19" s="16">
+        <f>L19+Drivers!M22</f>
+        <v/>
+      </c>
+      <c r="N19" s="16">
+        <f>M19+Drivers!N22</f>
+        <v/>
+      </c>
+      <c r="O19" s="16">
+        <f>N19+Drivers!O22</f>
+        <v/>
+      </c>
+      <c r="P19" s="16">
+        <f>O19+Drivers!P22</f>
+        <v/>
+      </c>
+      <c r="Q19" s="16">
+        <f>P19+Drivers!Q22</f>
+        <v/>
+      </c>
+      <c r="R19" s="16">
+        <f>Q19+Drivers!R22</f>
         <v/>
       </c>
     </row>
@@ -20442,7 +20542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20510,10 +20610,10 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2489.283062017579</v>
+        <v>2331.405852605007</v>
       </c>
       <c r="F2" t="n">
-        <v>1.921616198851587</v>
+        <v>1.934573376311912</v>
       </c>
       <c r="G2" t="n">
         <v>2.529091591591591</v>
@@ -20538,10 +20638,10 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2489.283062017579</v>
+        <v>2331.405852605007</v>
       </c>
       <c r="F3" t="n">
-        <v>1.921616198851587</v>
+        <v>1.934573376311912</v>
       </c>
       <c r="G3" t="n">
         <v>2.471612237237237</v>
@@ -20566,10 +20666,10 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>2489.283062017579</v>
+        <v>2331.405852605007</v>
       </c>
       <c r="F4" t="n">
-        <v>1.921616198851587</v>
+        <v>1.934573376311912</v>
       </c>
       <c r="G4" t="n">
         <v>2.6440503003003</v>
@@ -20588,22 +20688,22 @@
         <v>150</v>
       </c>
       <c r="C5" t="n">
-        <v>7200</v>
+        <v>8600</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>3856.179680289578</v>
+        <v>3550.376042067852</v>
       </c>
       <c r="F5" t="n">
-        <v>1.868248933488662</v>
+        <v>1.852526524148559</v>
       </c>
       <c r="G5" t="n">
-        <v>2.557643427741467</v>
+        <v>2.550336527492585</v>
       </c>
       <c r="H5" t="n">
-        <v>19.39591836734694</v>
+        <v>20.76734693877551</v>
       </c>
     </row>
     <row r="6">
@@ -20616,22 +20716,22 @@
         <v>300</v>
       </c>
       <c r="C6" t="n">
-        <v>11400</v>
+        <v>8600</v>
       </c>
       <c r="D6" t="n">
-        <v>2244.510174526423</v>
+        <v>2224.939741253336</v>
       </c>
       <c r="E6" t="n">
         <v>2000</v>
       </c>
       <c r="F6" t="n">
-        <v>1.860027494521559</v>
+        <v>1.908348056978604</v>
       </c>
       <c r="G6" t="n">
-        <v>2.498543123543123</v>
+        <v>2.50329038514824</v>
       </c>
       <c r="H6" t="n">
-        <v>35.85306122448979</v>
+        <v>33.11020408163265</v>
       </c>
     </row>
     <row r="7">
@@ -20647,7 +20747,7 @@
         <v>7000</v>
       </c>
       <c r="D7" t="n">
-        <v>2936.025161178578</v>
+        <v>3038.97007915886</v>
       </c>
       <c r="E7" t="n">
         <v>2000</v>
@@ -20678,10 +20778,10 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>4991.117838853224</v>
+        <v>4714.46836946547</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8232107028126554</v>
+        <v>0.8384681236346562</v>
       </c>
       <c r="G8" t="n">
         <v>1.671006944444444</v>
@@ -20703,13 +20803,13 @@
         <v>8600</v>
       </c>
       <c r="D9" t="n">
-        <v>201.5282692544952</v>
+        <v>348.9042746737423</v>
       </c>
       <c r="E9" t="n">
         <v>2000</v>
       </c>
       <c r="F9" t="n">
-        <v>2.12897004955669</v>
+        <v>2.129560851551169</v>
       </c>
       <c r="G9" t="n">
         <v>2.697697697697698</v>
@@ -20734,10 +20834,10 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>2900.711633446151</v>
+        <v>2733.191566890722</v>
       </c>
       <c r="F10" t="n">
-        <v>1.787319118465091</v>
+        <v>1.800467468286463</v>
       </c>
       <c r="G10" t="n">
         <v>2.427927927927928</v>
@@ -20762,10 +20862,10 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>2801.102610889759</v>
+        <v>2635.917130800497</v>
       </c>
       <c r="F11" t="n">
-        <v>1.818837821004778</v>
+        <v>1.831941303843456</v>
       </c>
       <c r="G11" t="n">
         <v>2.45167042042042</v>
@@ -20790,10 +20890,10 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>2291.797347731863</v>
+        <v>2138.548709747864</v>
       </c>
       <c r="F12" t="n">
-        <v>1.990135117416125</v>
+        <v>2.00299475795755</v>
       </c>
       <c r="G12" t="n">
         <v>2.580705705705705</v>
@@ -20815,7 +20915,7 @@
         <v>8600</v>
       </c>
       <c r="D13" t="n">
-        <v>2691.127201994906</v>
+        <v>2808.76599752621</v>
       </c>
       <c r="E13" t="n">
         <v>2000</v>
@@ -20846,10 +20946,10 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>4218.040612195502</v>
+        <v>4017.436029338358</v>
       </c>
       <c r="F14" t="n">
-        <v>1.311174924367514</v>
+        <v>1.325001067105324</v>
       </c>
       <c r="G14" t="n">
         <v>2.069256756756757</v>
@@ -20874,10 +20974,10 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>5444.988358677134</v>
+        <v>5272.781630448563</v>
       </c>
       <c r="F15" t="n">
-        <v>1.060671954326748</v>
+        <v>1.074967338314399</v>
       </c>
       <c r="G15" t="n">
         <v>1.820945945945946</v>
@@ -20899,7 +20999,7 @@
         <v>8600</v>
       </c>
       <c r="D16" t="n">
-        <v>6576.063417137786</v>
+        <v>6720.186302310181</v>
       </c>
       <c r="E16" t="n">
         <v>2000</v>
@@ -20927,7 +21027,7 @@
         <v>8600</v>
       </c>
       <c r="D17" t="n">
-        <v>6217.609994290794</v>
+        <v>6414.107963485019</v>
       </c>
       <c r="E17" t="n">
         <v>2000</v>
@@ -20958,10 +21058,10 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>6319.750536277137</v>
+        <v>6198.606734848563</v>
       </c>
       <c r="F18" t="n">
-        <v>1.479614443006876</v>
+        <v>1.490994927161221</v>
       </c>
       <c r="G18" t="n">
         <v>1.896818693693693</v>
@@ -20986,10 +21086,10 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>4280.86217892523</v>
+        <v>4096.771783946659</v>
       </c>
       <c r="F19" t="n">
-        <v>1.667673513120401</v>
+        <v>1.682132262326544</v>
       </c>
       <c r="G19" t="n">
         <v>2.529091591591591</v>
@@ -21011,13 +21111,13 @@
         <v>8600</v>
       </c>
       <c r="D20" t="n">
-        <v>3466.95484215277</v>
+        <v>3617.321806234756</v>
       </c>
       <c r="E20" t="n">
         <v>2000</v>
       </c>
       <c r="F20" t="n">
-        <v>2.032113867380101</v>
+        <v>2.032790391171389</v>
       </c>
       <c r="G20" t="n">
         <v>2.529091591591591</v>
@@ -21039,13 +21139,13 @@
         <v>8600</v>
       </c>
       <c r="D21" t="n">
-        <v>3592.738304119634</v>
+        <v>3758.30389207087</v>
       </c>
       <c r="E21" t="n">
         <v>2000</v>
       </c>
       <c r="F21" t="n">
-        <v>2.029467523767343</v>
+        <v>2.029735897096021</v>
       </c>
       <c r="G21" t="n">
         <v>2.529091591591591</v>
@@ -21070,10 +21170,10 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>5493.550816277133</v>
+        <v>5344.374804848561</v>
       </c>
       <c r="F22" t="n">
-        <v>1.538420503155891</v>
+        <v>1.551377680616217</v>
       </c>
       <c r="G22" t="n">
         <v>2.529091591591591</v>
@@ -21098,10 +21198,10 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>2761.332812017578</v>
+        <v>2599.705602605006</v>
       </c>
       <c r="F23" t="n">
-        <v>1.886083036783268</v>
+        <v>1.899327611015366</v>
       </c>
       <c r="G23" t="n">
         <v>2.529091591591591</v>
@@ -21123,13 +21223,13 @@
         <v>8600</v>
       </c>
       <c r="D24" t="n">
-        <v>411.8212896626601</v>
+        <v>562.4115807961907</v>
       </c>
       <c r="E24" t="n">
         <v>2000</v>
       </c>
       <c r="F24" t="n">
-        <v>1.996654055937625</v>
+        <v>1.997207932807449</v>
       </c>
       <c r="G24" t="n">
         <v>2.529091591591591</v>
@@ -21151,7 +21251,7 @@
         <v>8600</v>
       </c>
       <c r="D25" t="n">
-        <v>8277.861895872455</v>
+        <v>8450.679262832331</v>
       </c>
       <c r="E25" t="n">
         <v>2000</v>
@@ -21182,10 +21282,10 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>8615.757459183675</v>
+        <v>8132.543173469388</v>
       </c>
       <c r="F26" t="n">
-        <v>1.959935768421156</v>
+        <v>1.972318152337938</v>
       </c>
       <c r="G26" t="n">
         <v>2.529091591591591</v>
@@ -21210,10 +21310,10 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>2489.283062017579</v>
+        <v>2331.405852605007</v>
       </c>
       <c r="F27" t="n">
-        <v>1.921616198851587</v>
+        <v>1.934573376311912</v>
       </c>
       <c r="G27" t="n">
         <v>2.529091591591591</v>
@@ -21235,19 +21335,131 @@
         <v>8600</v>
       </c>
       <c r="D28" t="n">
-        <v>1510.716937982421</v>
+        <v>1668.594147394994</v>
       </c>
       <c r="E28" t="n">
         <v>4000</v>
       </c>
       <c r="F28" t="n">
-        <v>1.805836153241698</v>
+        <v>1.806693757282954</v>
       </c>
       <c r="G28" t="n">
         <v>2.529091591591591</v>
       </c>
       <c r="H28" t="n">
         <v>24.88163265306122</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>mw_added_2026q3 = 25</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>25</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8250</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2353.849121626719</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.943009884783294</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2.530270655270655</v>
+      </c>
+      <c r="H29" t="n">
+        <v>24.53877551020408</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>mw_added_2026q3 = 200</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>200</v>
+      </c>
+      <c r="C30" t="n">
+        <v>10700</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2182.074075667853</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.887866523418304</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2.522563967753242</v>
+      </c>
+      <c r="H30" t="n">
+        <v>26.93877551020408</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mw_added_2026q4 = 200</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>200</v>
+      </c>
+      <c r="C31" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2553.740033334093</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.97446700481743</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2.536616161616161</v>
+      </c>
+      <c r="H31" t="n">
+        <v>22.82448979591836</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>mw_added_2026q4 = 500</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>500</v>
+      </c>
+      <c r="C32" t="n">
+        <v>10700</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2028.412910639283</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.899965338964854</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2.522563967753242</v>
+      </c>
+      <c r="H32" t="n">
+        <v>26.93877551020408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>